<commit_message>
fix: update the content
</commit_message>
<xml_diff>
--- a/result/organelle_protein_abundance_ecGEMs.xlsx
+++ b/result/organelle_protein_abundance_ecGEMs.xlsx
@@ -517,13 +517,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.002789089909112443</v>
+        <v>0.002789089909112446</v>
       </c>
       <c r="C2" t="n">
-        <v>0.002100510462592406</v>
+        <v>0.002100510462592407</v>
       </c>
       <c r="D2" t="n">
-        <v>0.001517172110086583</v>
+        <v>0.001517172110086582</v>
       </c>
       <c r="E2" t="n">
         <v>0.0004081038291541514</v>
@@ -532,7 +532,7 @@
         <v>0.001002817663262919</v>
       </c>
       <c r="G2" t="n">
-        <v>5.641755796595917e-05</v>
+        <v>5.641755796595914e-05</v>
       </c>
       <c r="H2" t="n">
         <v>0.0001034452159839899</v>
@@ -550,7 +550,7 @@
         <v>1.537639383823591e-05</v>
       </c>
       <c r="M2" t="n">
-        <v>8.370334948974562e-06</v>
+        <v>8.37033494897456e-06</v>
       </c>
       <c r="N2" t="n">
         <v>1.575149012347947e-06</v>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.003261946963489568</v>
+        <v>0.003261946963489564</v>
       </c>
       <c r="C3" t="n">
         <v>0.001895046452360417</v>
@@ -587,7 +587,7 @@
         <v>0.0006602698876797595</v>
       </c>
       <c r="G3" t="n">
-        <v>6.099841607543444e-05</v>
+        <v>6.099841607543441e-05</v>
       </c>
       <c r="H3" t="n">
         <v>0.0003614122715047945</v>
@@ -599,7 +599,7 @@
         <v>4.566102358580122e-05</v>
       </c>
       <c r="K3" t="n">
-        <v>2.865075060407798e-05</v>
+        <v>2.865075060407797e-05</v>
       </c>
       <c r="L3" t="n">
         <v>4.495314657295621e-05</v>
@@ -627,22 +627,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.002985435584777134</v>
+        <v>0.002985435584777132</v>
       </c>
       <c r="C4" t="n">
         <v>0.001485149893287112</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0007910250416219663</v>
+        <v>0.0007910250416219666</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0003307900569942437</v>
+        <v>0.0003307900569942438</v>
       </c>
       <c r="F4" t="n">
         <v>0.0003391161071029701</v>
       </c>
       <c r="G4" t="n">
-        <v>6.591100920985533e-05</v>
+        <v>6.591100920985532e-05</v>
       </c>
       <c r="H4" t="n">
         <v>0.0001897398077763376</v>
@@ -654,7 +654,7 @@
         <v>5.045299211077879e-05</v>
       </c>
       <c r="K4" t="n">
-        <v>4.252440093195754e-05</v>
+        <v>4.252440093195753e-05</v>
       </c>
       <c r="L4" t="n">
         <v>0.0001009189846054253</v>
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.002196174576519605</v>
+        <v>0.002196174576519606</v>
       </c>
       <c r="C5" t="n">
         <v>0.001548311062317886</v>
       </c>
       <c r="D5" t="n">
-        <v>0.001018370535335372</v>
+        <v>0.001018370535335371</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0004408599331625325</v>
+        <v>0.0004408599331625326</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0003641652263605138</v>
+        <v>0.0003641652263605139</v>
       </c>
       <c r="G5" t="n">
         <v>0.0001217842236043435</v>
@@ -721,7 +721,7 @@
         <v>6.156936170388864e-06</v>
       </c>
       <c r="O5" t="n">
-        <v>8.005476573417074e-07</v>
+        <v>8.005476573417073e-07</v>
       </c>
       <c r="P5" t="n">
         <v>1.945758491311669e-07</v>
@@ -743,7 +743,7 @@
         <v>0.0008271428933847369</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0006809576837215202</v>
+        <v>0.0006809576837215199</v>
       </c>
       <c r="E6" t="n">
         <v>0.000140902108719196</v>
@@ -752,7 +752,7 @@
         <v>0.000230424621062976</v>
       </c>
       <c r="G6" t="n">
-        <v>4.702804620304099e-05</v>
+        <v>4.702804620304102e-05</v>
       </c>
       <c r="H6" t="n">
         <v>3.721176535657498e-05</v>
@@ -764,10 +764,10 @@
         <v>1.9107333851922e-05</v>
       </c>
       <c r="K6" t="n">
-        <v>2.278488857891e-05</v>
+        <v>2.278488857891001e-05</v>
       </c>
       <c r="L6" t="n">
-        <v>8.153574401448999e-06</v>
+        <v>8.153574401449e-06</v>
       </c>
       <c r="M6" t="n">
         <v>4.807132404725e-06</v>
@@ -795,7 +795,7 @@
         <v>0.001628162641109837</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0008645439839577341</v>
+        <v>0.000864543983957734</v>
       </c>
       <c r="D7" t="n">
         <v>0.0007413553883853359</v>
@@ -804,16 +804,16 @@
         <v>0.000106308355953004</v>
       </c>
       <c r="F7" t="n">
-        <v>0.000247830266770496</v>
+        <v>0.0002478302667704959</v>
       </c>
       <c r="G7" t="n">
-        <v>6.267239897635701e-05</v>
+        <v>6.2672398976357e-05</v>
       </c>
       <c r="H7" t="n">
         <v>5.786227247874898e-05</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0001677574470930019</v>
+        <v>0.000167757447093002</v>
       </c>
       <c r="J7" t="n">
         <v>2.889705412265801e-05</v>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001424243781485717</v>
+        <v>0.001424243781485716</v>
       </c>
       <c r="C8" t="n">
-        <v>0.000772263012191321</v>
+        <v>0.0007722630121913211</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0006777698786108077</v>
+        <v>0.0006777698786108076</v>
       </c>
       <c r="E8" t="n">
         <v>8.660382070493401e-05</v>
@@ -862,13 +862,13 @@
         <v>0.00020787930207662</v>
       </c>
       <c r="G8" t="n">
-        <v>5.423355403242101e-05</v>
+        <v>5.423355403242103e-05</v>
       </c>
       <c r="H8" t="n">
         <v>4.9459221464865e-05</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0001419080703416919</v>
+        <v>0.000141908070341692</v>
       </c>
       <c r="J8" t="n">
         <v>2.474333099120901e-05</v>
@@ -877,13 +877,13 @@
         <v>2.016101826924e-05</v>
       </c>
       <c r="L8" t="n">
-        <v>8.305856010314001e-06</v>
+        <v>8.305856010313999e-06</v>
       </c>
       <c r="M8" t="n">
         <v>5.644894063427e-06</v>
       </c>
       <c r="N8" t="n">
-        <v>7.449025653120002e-07</v>
+        <v>7.449025653120001e-07</v>
       </c>
       <c r="O8" t="n">
         <v>1.49354964347e-07</v>
@@ -902,13 +902,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001426433783978344</v>
+        <v>0.001426433783978345</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0007355408626357024</v>
+        <v>0.0007355408626357019</v>
       </c>
       <c r="D9" t="n">
-        <v>0.000648863878355667</v>
+        <v>0.0006488638783556673</v>
       </c>
       <c r="E9" t="n">
         <v>8.7161569886248e-05</v>
@@ -917,7 +917,7 @@
         <v>0.000194493425280166</v>
       </c>
       <c r="G9" t="n">
-        <v>5.4126547565832e-05</v>
+        <v>5.412654756583202e-05</v>
       </c>
       <c r="H9" t="n">
         <v>5.188366716982499e-05</v>
@@ -935,10 +935,10 @@
         <v>9.138060582981001e-06</v>
       </c>
       <c r="M9" t="n">
-        <v>5.828014403199e-06</v>
+        <v>5.828014403199001e-06</v>
       </c>
       <c r="N9" t="n">
-        <v>7.78252690495e-07</v>
+        <v>7.782526904950001e-07</v>
       </c>
       <c r="O9" t="n">
         <v>1.63665956998e-07</v>
@@ -957,19 +957,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.001394776382373676</v>
+        <v>0.001394776382373677</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0006535386756523972</v>
+        <v>0.0006535386756523969</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0005996363158010768</v>
+        <v>0.0005996363158010773</v>
       </c>
       <c r="E10" t="n">
         <v>8.293966947341201e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0001647535216536201</v>
+        <v>0.00016475352165362</v>
       </c>
       <c r="G10" t="n">
         <v>5.9706825725492e-05</v>
@@ -984,7 +984,7 @@
         <v>2.9419623817777e-05</v>
       </c>
       <c r="K10" t="n">
-        <v>2.2147184484e-05</v>
+        <v>2.214718448400001e-05</v>
       </c>
       <c r="L10" t="n">
         <v>1.0000807346547e-05</v>
@@ -993,7 +993,7 @@
         <v>5.887135652105999e-06</v>
       </c>
       <c r="N10" t="n">
-        <v>9.345764390590001e-07</v>
+        <v>9.34576439059e-07</v>
       </c>
       <c r="O10" t="n">
         <v>1.76856388858e-07</v>
@@ -1012,22 +1012,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00139565184923646</v>
+        <v>0.001395651849236461</v>
       </c>
       <c r="C11" t="n">
-        <v>0.000693355697908238</v>
+        <v>0.0006933556979082377</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0006298683277803272</v>
+        <v>0.0006298683277803271</v>
       </c>
       <c r="E11" t="n">
-        <v>8.327862934156099e-05</v>
+        <v>8.3278629341561e-05</v>
       </c>
       <c r="F11" t="n">
         <v>0.000185381544645871</v>
       </c>
       <c r="G11" t="n">
-        <v>5.489949164330601e-05</v>
+        <v>5.489949164330599e-05</v>
       </c>
       <c r="H11" t="n">
         <v>5.012157435197999e-05</v>
@@ -1048,7 +1048,7 @@
         <v>5.90181297781e-06</v>
       </c>
       <c r="N11" t="n">
-        <v>8.434846144460001e-07</v>
+        <v>8.434846144459998e-07</v>
       </c>
       <c r="O11" t="n">
         <v>1.7953978041e-07</v>
@@ -1070,19 +1070,19 @@
         <v>0.001478727074812343</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0007202914127668788</v>
+        <v>0.0007202914127668786</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0006729246035505318</v>
+        <v>0.0006729246035505319</v>
       </c>
       <c r="E12" t="n">
-        <v>8.656312844023098e-05</v>
+        <v>8.656312844023099e-05</v>
       </c>
       <c r="F12" t="n">
         <v>0.000160529967346987</v>
       </c>
       <c r="G12" t="n">
-        <v>5.932642877221302e-05</v>
+        <v>5.9326428772213e-05</v>
       </c>
       <c r="H12" t="n">
         <v>5.550375985464803e-05</v>
@@ -1103,7 +1103,7 @@
         <v>6.014676826820001e-06</v>
       </c>
       <c r="N12" t="n">
-        <v>8.817635708130001e-07</v>
+        <v>8.81763570813e-07</v>
       </c>
       <c r="O12" t="n">
         <v>1.79243159899e-07</v>
@@ -1122,19 +1122,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.002091681617060734</v>
+        <v>0.002091681617060732</v>
       </c>
       <c r="C13" t="n">
         <v>0.001131153614807681</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0009472159598732002</v>
+        <v>0.0009472159598732</v>
       </c>
       <c r="E13" t="n">
         <v>0.000168851553251448</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0003161348123276611</v>
+        <v>0.000316134812327661</v>
       </c>
       <c r="G13" t="n">
         <v>7.307995132909099e-05</v>
@@ -1155,7 +1155,7 @@
         <v>1.1371804717243e-05</v>
       </c>
       <c r="M13" t="n">
-        <v>7.334028862789999e-06</v>
+        <v>7.334028862790001e-06</v>
       </c>
       <c r="N13" t="n">
         <v>1.273164906155e-06</v>
@@ -1180,10 +1180,10 @@
         <v>0.002130349303924622</v>
       </c>
       <c r="C14" t="n">
-        <v>0.001144495394398213</v>
+        <v>0.001144495394398214</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0009552340755060922</v>
+        <v>0.0009552340755060913</v>
       </c>
       <c r="E14" t="n">
         <v>0.000162577172017433</v>
@@ -1192,7 +1192,7 @@
         <v>0.00032821944206928</v>
       </c>
       <c r="G14" t="n">
-        <v>7.627272152385499e-05</v>
+        <v>7.627272152385504e-05</v>
       </c>
       <c r="H14" t="n">
         <v>6.1505023995093e-05</v>
@@ -1210,7 +1210,7 @@
         <v>1.2655029607194e-05</v>
       </c>
       <c r="M14" t="n">
-        <v>7.070972685420001e-06</v>
+        <v>7.07097268542e-06</v>
       </c>
       <c r="N14" t="n">
         <v>1.325115395667e-06</v>
@@ -1238,7 +1238,7 @@
         <v>0.001074373258554613</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0008935516315664512</v>
+        <v>0.000893551631566451</v>
       </c>
       <c r="E15" t="n">
         <v>0.000165940291696469</v>
@@ -1253,7 +1253,7 @@
         <v>6.565670927224401e-05</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0001928777418990781</v>
+        <v>0.000192877741899078</v>
       </c>
       <c r="J15" t="n">
         <v>3.933027755412599e-05</v>
@@ -1287,10 +1287,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.002337050695204704</v>
+        <v>0.002337050695204707</v>
       </c>
       <c r="C16" t="n">
-        <v>0.00138586832278534</v>
+        <v>0.001385868322785341</v>
       </c>
       <c r="D16" t="n">
         <v>0.001092349573714423</v>
@@ -1302,7 +1302,7 @@
         <v>0.000417776804976858</v>
       </c>
       <c r="G16" t="n">
-        <v>7.952773957951295e-05</v>
+        <v>7.952773957951301e-05</v>
       </c>
       <c r="H16" t="n">
         <v>6.942122357119901e-05</v>
@@ -1345,10 +1345,10 @@
         <v>0.001389921121527817</v>
       </c>
       <c r="C17" t="n">
-        <v>0.000702731298572263</v>
+        <v>0.0007027312985722629</v>
       </c>
       <c r="D17" t="n">
-        <v>0.000604173884546236</v>
+        <v>0.0006041738845462363</v>
       </c>
       <c r="E17" t="n">
         <v>0.00012907891924807</v>
@@ -1357,13 +1357,13 @@
         <v>0.000182177389886671</v>
       </c>
       <c r="G17" t="n">
-        <v>4.206631544844699e-05</v>
+        <v>4.206631544844701e-05</v>
       </c>
       <c r="H17" t="n">
         <v>3.1721285806796e-05</v>
       </c>
       <c r="I17" t="n">
-        <v>9.440182293646301e-05</v>
+        <v>9.4401822936463e-05</v>
       </c>
       <c r="J17" t="n">
         <v>1.7512137935244e-05</v>
@@ -1372,13 +1372,13 @@
         <v>2.081565595782e-05</v>
       </c>
       <c r="L17" t="n">
-        <v>7.557336071243e-06</v>
+        <v>7.557336071243001e-06</v>
       </c>
       <c r="M17" t="n">
         <v>4.091763683615e-06</v>
       </c>
       <c r="N17" t="n">
-        <v>6.09807433796e-07</v>
+        <v>6.098074337959999e-07</v>
       </c>
       <c r="O17" t="n">
         <v>1.69666332621e-07</v>
@@ -1406,10 +1406,10 @@
         <v>0.001177051307197048</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0002545628961365729</v>
+        <v>0.000254562896136573</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0005500204697614171</v>
+        <v>0.000550020469761417</v>
       </c>
       <c r="G18" t="n">
         <v>8.285085269981502e-05</v>
@@ -1424,7 +1424,7 @@
         <v>4.651149162087001e-05</v>
       </c>
       <c r="K18" t="n">
-        <v>2.727377272881e-05</v>
+        <v>2.727377272881001e-05</v>
       </c>
       <c r="L18" t="n">
         <v>1.2001970380439e-05</v>
@@ -1452,13 +1452,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.002483024743292037</v>
+        <v>0.002483024743292039</v>
       </c>
       <c r="C19" t="n">
-        <v>0.001426624510038333</v>
+        <v>0.001426624510038332</v>
       </c>
       <c r="D19" t="n">
-        <v>0.001091168343543609</v>
+        <v>0.001091168343543608</v>
       </c>
       <c r="E19" t="n">
         <v>0.000252772489320358</v>
@@ -1467,13 +1467,13 @@
         <v>0.000447085185179899</v>
       </c>
       <c r="G19" t="n">
-        <v>8.585308601595e-05</v>
+        <v>8.585308601595001e-05</v>
       </c>
       <c r="H19" t="n">
         <v>7.492777240859499e-05</v>
       </c>
       <c r="I19" t="n">
-        <v>0.000249970770223323</v>
+        <v>0.0002499707702233231</v>
       </c>
       <c r="J19" t="n">
         <v>4.694084140522601e-05</v>
@@ -1507,22 +1507,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.002647579501936081</v>
+        <v>0.002647579501936082</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0012960407681084</v>
+        <v>0.001296040768108399</v>
       </c>
       <c r="D20" t="n">
         <v>0.001162764740028258</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0003123861398319071</v>
+        <v>0.000312386139831907</v>
       </c>
       <c r="F20" t="n">
         <v>0.000143804709886088</v>
       </c>
       <c r="G20" t="n">
-        <v>7.301924023777101e-05</v>
+        <v>7.301924023777096e-05</v>
       </c>
       <c r="H20" t="n">
         <v>3.466016598811299e-05</v>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.003075047430155734</v>
+        <v>0.003075047430155733</v>
       </c>
       <c r="C21" t="n">
         <v>0.001439605898713449</v>
@@ -1571,13 +1571,13 @@
         <v>0.001426336267504667</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0002958668963129081</v>
+        <v>0.000295866896312908</v>
       </c>
       <c r="F21" t="n">
         <v>0.000194720354163909</v>
       </c>
       <c r="G21" t="n">
-        <v>9.489105559325198e-05</v>
+        <v>9.4891055593252e-05</v>
       </c>
       <c r="H21" t="n">
         <v>4.513851306233402e-05</v>
@@ -1595,7 +1595,7 @@
         <v>1.5152773335726e-05</v>
       </c>
       <c r="M21" t="n">
-        <v>9.25510768312e-06</v>
+        <v>9.255107683120001e-06</v>
       </c>
       <c r="N21" t="n">
         <v>1.992668576019e-06</v>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.003165996751038781</v>
+        <v>0.00316599675103878</v>
       </c>
       <c r="C22" t="n">
         <v>0.001587001811470749</v>
@@ -1632,7 +1632,7 @@
         <v>0.000240556811909469</v>
       </c>
       <c r="G22" t="n">
-        <v>8.372940859978299e-05</v>
+        <v>8.372940859978294e-05</v>
       </c>
       <c r="H22" t="n">
         <v>5.318177738814198e-05</v>
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.002750579116873123</v>
+        <v>0.002750579116873124</v>
       </c>
       <c r="C23" t="n">
         <v>0.001220731697980852</v>
@@ -1681,25 +1681,25 @@
         <v>0.001229009438949799</v>
       </c>
       <c r="E23" t="n">
-        <v>0.000233754460725607</v>
+        <v>0.0002337544607256071</v>
       </c>
       <c r="F23" t="n">
         <v>0.0002661256332602969</v>
       </c>
       <c r="G23" t="n">
-        <v>6.999202738920301e-05</v>
+        <v>6.999202738920304e-05</v>
       </c>
       <c r="H23" t="n">
         <v>4.854447758271501e-05</v>
       </c>
       <c r="I23" t="n">
-        <v>0.0002642275592367051</v>
+        <v>0.000264227559236705</v>
       </c>
       <c r="J23" t="n">
         <v>3.1205054563452e-05</v>
       </c>
       <c r="K23" t="n">
-        <v>3.799569493278e-05</v>
+        <v>3.799569493278001e-05</v>
       </c>
       <c r="L23" t="n">
         <v>1.4302831053679e-05</v>
@@ -1730,10 +1730,10 @@
         <v>0.001718766626401084</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0008608978806600518</v>
+        <v>0.0008608978806600519</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0006511368885527281</v>
+        <v>0.0006511368885527276</v>
       </c>
       <c r="E24" t="n">
         <v>0.000175216221285004</v>
@@ -1763,7 +1763,7 @@
         <v>6.05010852511e-06</v>
       </c>
       <c r="N24" t="n">
-        <v>7.94214228791e-07</v>
+        <v>7.942142287909999e-07</v>
       </c>
       <c r="O24" t="n">
         <v>1.7905791382e-07</v>
@@ -1785,19 +1785,19 @@
         <v>0.002174994579390263</v>
       </c>
       <c r="C25" t="n">
-        <v>0.001132000459232332</v>
+        <v>0.001132000459232331</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0008634413394306489</v>
+        <v>0.000863441339430649</v>
       </c>
       <c r="E25" t="n">
         <v>0.000233197437768465</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0002954333852870631</v>
+        <v>0.0002954333852870629</v>
       </c>
       <c r="G25" t="n">
-        <v>5.119281883165802e-05</v>
+        <v>5.1192818831658e-05</v>
       </c>
       <c r="H25" t="n">
         <v>3.481611368004601e-05</v>
@@ -1818,7 +1818,7 @@
         <v>7.29429967016e-06</v>
       </c>
       <c r="N25" t="n">
-        <v>8.681844018569999e-07</v>
+        <v>8.681844018570002e-07</v>
       </c>
       <c r="O25" t="n">
         <v>2.09128266658e-07</v>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.001187508468748142</v>
+        <v>0.001187508468748141</v>
       </c>
       <c r="C26" t="n">
         <v>0.0006214545978980252</v>
@@ -1846,13 +1846,13 @@
         <v>0.000481476391599704</v>
       </c>
       <c r="E26" t="n">
-        <v>7.076641610926601e-05</v>
+        <v>7.0766416109266e-05</v>
       </c>
       <c r="F26" t="n">
         <v>0.000212120710794537</v>
       </c>
       <c r="G26" t="n">
-        <v>4.396550077436499e-05</v>
+        <v>4.396550077436501e-05</v>
       </c>
       <c r="H26" t="n">
         <v>3.539994858749199e-05</v>
@@ -1867,7 +1867,7 @@
         <v>1.733077167569e-05</v>
       </c>
       <c r="L26" t="n">
-        <v>8.575640102151e-06</v>
+        <v>8.575640102150999e-06</v>
       </c>
       <c r="M26" t="n">
         <v>4.213426341117e-06</v>
@@ -1892,22 +1892,22 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.001975801108823517</v>
+        <v>0.001975801108823518</v>
       </c>
       <c r="C27" t="n">
-        <v>0.0009800356943220141</v>
+        <v>0.0009800356943220139</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0008160191779724464</v>
+        <v>0.0008160191779724462</v>
       </c>
       <c r="E27" t="n">
         <v>0.000117428810539258</v>
       </c>
       <c r="F27" t="n">
-        <v>0.000317874080746215</v>
+        <v>0.0003178740807462151</v>
       </c>
       <c r="G27" t="n">
-        <v>7.1741558764523e-05</v>
+        <v>7.174155876452299e-05</v>
       </c>
       <c r="H27" t="n">
         <v>5.775404506387601e-05</v>
@@ -1925,7 +1925,7 @@
         <v>1.292023536781e-05</v>
       </c>
       <c r="M27" t="n">
-        <v>6.98274094302e-06</v>
+        <v>6.982740943020001e-06</v>
       </c>
       <c r="N27" t="n">
         <v>1.001031194059e-06</v>
@@ -1950,10 +1950,10 @@
         <v>0.001460744581266093</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0007419273006867911</v>
+        <v>0.0007419273006867909</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0006699175509989459</v>
+        <v>0.0006699175509989457</v>
       </c>
       <c r="E28" t="n">
         <v>0.000122909151025617</v>
@@ -1962,13 +1962,13 @@
         <v>0.000154706249773661</v>
       </c>
       <c r="G28" t="n">
-        <v>4.385525491902499e-05</v>
+        <v>4.3855254919025e-05</v>
       </c>
       <c r="H28" t="n">
         <v>3.5622229652718e-05</v>
       </c>
       <c r="I28" t="n">
-        <v>9.873062316118202e-05</v>
+        <v>9.8730623161182e-05</v>
       </c>
       <c r="J28" t="n">
         <v>1.7918686272561e-05</v>
@@ -1977,7 +1977,7 @@
         <v>2.109781657208e-05</v>
       </c>
       <c r="L28" t="n">
-        <v>7.54942784943e-06</v>
+        <v>7.549427849429999e-06</v>
       </c>
       <c r="M28" t="n">
         <v>4.10400489123e-06</v>
@@ -2002,22 +2002,22 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.001918146401735119</v>
+        <v>0.001918146401735118</v>
       </c>
       <c r="C29" t="n">
-        <v>0.0009073322106913279</v>
+        <v>0.0009073322106913281</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0008166917101082262</v>
+        <v>0.0008166917101082256</v>
       </c>
       <c r="E29" t="n">
         <v>0.000116169264681899</v>
       </c>
       <c r="F29" t="n">
-        <v>0.000255005321983555</v>
+        <v>0.0002550053219835551</v>
       </c>
       <c r="G29" t="n">
-        <v>7.168979976017901e-05</v>
+        <v>7.168979976017899e-05</v>
       </c>
       <c r="H29" t="n">
         <v>5.5720659876872e-05</v>
@@ -2029,13 +2029,13 @@
         <v>3.0744602016985e-05</v>
       </c>
       <c r="K29" t="n">
-        <v>2.846595181169e-05</v>
+        <v>2.846595181168999e-05</v>
       </c>
       <c r="L29" t="n">
         <v>1.2267651928845e-05</v>
       </c>
       <c r="M29" t="n">
-        <v>7.300385063530001e-06</v>
+        <v>7.30038506353e-06</v>
       </c>
       <c r="N29" t="n">
         <v>1.011034670357e-06</v>
@@ -2057,13 +2057,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.002279597035932454</v>
+        <v>0.002279597035932452</v>
       </c>
       <c r="C30" t="n">
-        <v>0.0009230735426019359</v>
+        <v>0.0009230735426019358</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0009671104444196924</v>
+        <v>0.000967110444419692</v>
       </c>
       <c r="E30" t="n">
         <v>0.000100528108785147</v>
@@ -2072,7 +2072,7 @@
         <v>0.000186335899768822</v>
       </c>
       <c r="G30" t="n">
-        <v>6.596195673841102e-05</v>
+        <v>6.596195673841098e-05</v>
       </c>
       <c r="H30" t="n">
         <v>2.766917342503e-05</v>
@@ -2127,13 +2127,13 @@
         <v>0.000195272497187265</v>
       </c>
       <c r="G31" t="n">
-        <v>6.899498619751201e-05</v>
+        <v>6.899498619751198e-05</v>
       </c>
       <c r="H31" t="n">
         <v>3.5779596676096e-05</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0002675931268734419</v>
+        <v>0.000267593126873442</v>
       </c>
       <c r="J31" t="n">
         <v>3.1591158982887e-05</v>
@@ -2145,7 +2145,7 @@
         <v>2.2009005370587e-05</v>
       </c>
       <c r="M31" t="n">
-        <v>7.89436142823e-06</v>
+        <v>7.894361428229999e-06</v>
       </c>
       <c r="N31" t="n">
         <v>1.365427420157e-06</v>
@@ -2167,13 +2167,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.002403471768803232</v>
+        <v>0.002403471768803231</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0009445412445032146</v>
+        <v>0.0009445412445032151</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0009762795871151673</v>
+        <v>0.0009762795871151676</v>
       </c>
       <c r="E32" t="n">
         <v>0.000109320887182249</v>
@@ -2182,7 +2182,7 @@
         <v>0.000184172536277603</v>
       </c>
       <c r="G32" t="n">
-        <v>6.030654040334997e-05</v>
+        <v>6.030654040334999e-05</v>
       </c>
       <c r="H32" t="n">
         <v>3.3521442760779e-05</v>
@@ -2194,7 +2194,7 @@
         <v>2.901297643093001e-05</v>
       </c>
       <c r="K32" t="n">
-        <v>4.297465657065001e-05</v>
+        <v>4.297465657065e-05</v>
       </c>
       <c r="L32" t="n">
         <v>2.0913121960668e-05</v>
@@ -2237,7 +2237,7 @@
         <v>0.000272974410633343</v>
       </c>
       <c r="G33" t="n">
-        <v>8.332788092700899e-05</v>
+        <v>8.332788092700896e-05</v>
       </c>
       <c r="H33" t="n">
         <v>6.576947149348401e-05</v>
@@ -2249,7 +2249,7 @@
         <v>3.6609589946338e-05</v>
       </c>
       <c r="K33" t="n">
-        <v>3.299725525757e-05</v>
+        <v>3.299725525757001e-05</v>
       </c>
       <c r="L33" t="n">
         <v>1.390121227729e-05</v>
@@ -2277,13 +2277,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.002087573838834057</v>
+        <v>0.002087573838834056</v>
       </c>
       <c r="C34" t="n">
         <v>0.001003592182808837</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0008676597859003032</v>
+        <v>0.000867659785900303</v>
       </c>
       <c r="E34" t="n">
         <v>0.000116346213647287</v>
@@ -2292,7 +2292,7 @@
         <v>0.0002856913005182341</v>
       </c>
       <c r="G34" t="n">
-        <v>7.621242931865002e-05</v>
+        <v>7.621242931864997e-05</v>
       </c>
       <c r="H34" t="n">
         <v>5.986906439398401e-05</v>
@@ -2332,13 +2332,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.002130994005406564</v>
+        <v>0.002130994005406565</v>
       </c>
       <c r="C35" t="n">
-        <v>0.0009685390031590709</v>
+        <v>0.0009685390031590707</v>
       </c>
       <c r="D35" t="n">
-        <v>0.000848325521232799</v>
+        <v>0.0008483255212327988</v>
       </c>
       <c r="E35" t="n">
         <v>0.000115348799750992</v>
@@ -2347,13 +2347,13 @@
         <v>0.000293457389692407</v>
       </c>
       <c r="G35" t="n">
-        <v>8.1598036057091e-05</v>
+        <v>8.159803605709099e-05</v>
       </c>
       <c r="H35" t="n">
         <v>6.481736414871402e-05</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0002536559719695011</v>
+        <v>0.000253655971969501</v>
       </c>
       <c r="J35" t="n">
         <v>3.456112410101801e-05</v>
@@ -2365,7 +2365,7 @@
         <v>1.2470874564821e-05</v>
       </c>
       <c r="M35" t="n">
-        <v>7.996735338889998e-06</v>
+        <v>7.996735338890001e-06</v>
       </c>
       <c r="N35" t="n">
         <v>1.225609693245e-06</v>
@@ -2387,13 +2387,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.001779320199232576</v>
+        <v>0.001779320199232575</v>
       </c>
       <c r="C36" t="n">
         <v>0.0007971455345354092</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0006536127986632184</v>
+        <v>0.0006536127986632179</v>
       </c>
       <c r="E36" t="n">
         <v>0.000160970876134667</v>
@@ -2402,7 +2402,7 @@
         <v>0.000193066783719742</v>
       </c>
       <c r="G36" t="n">
-        <v>4.552391314210603e-05</v>
+        <v>4.552391314210601e-05</v>
       </c>
       <c r="H36" t="n">
         <v>3.188748124522699e-05</v>
@@ -2423,7 +2423,7 @@
         <v>6.13367583555e-06</v>
       </c>
       <c r="N36" t="n">
-        <v>8.354525352670001e-07</v>
+        <v>8.35452535267e-07</v>
       </c>
       <c r="O36" t="n">
         <v>2.15344543845e-07</v>
@@ -2442,13 +2442,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.002229780770924003</v>
+        <v>0.002229780770924002</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0009464258153049811</v>
+        <v>0.0009464258153049808</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0009320673566888116</v>
+        <v>0.0009320673566888113</v>
       </c>
       <c r="E37" t="n">
         <v>0.000170673908880417</v>
@@ -2457,25 +2457,25 @@
         <v>0.000216004150208319</v>
       </c>
       <c r="G37" t="n">
-        <v>6.649284948718601e-05</v>
+        <v>6.649284948718602e-05</v>
       </c>
       <c r="H37" t="n">
         <v>3.941772701123597e-05</v>
       </c>
       <c r="I37" t="n">
-        <v>0.000219416615028068</v>
+        <v>0.0002194166150280681</v>
       </c>
       <c r="J37" t="n">
         <v>2.7010563575516e-05</v>
       </c>
       <c r="K37" t="n">
-        <v>3.325092764549001e-05</v>
+        <v>3.325092764548999e-05</v>
       </c>
       <c r="L37" t="n">
         <v>1.1131725715406e-05</v>
       </c>
       <c r="M37" t="n">
-        <v>7.49437458636e-06</v>
+        <v>7.494374586360001e-06</v>
       </c>
       <c r="N37" t="n">
         <v>1.225981368802e-06</v>
@@ -2497,22 +2497,22 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.002014272657407696</v>
+        <v>0.002014272657407697</v>
       </c>
       <c r="C38" t="n">
         <v>0.001032100836786488</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0006970971927042915</v>
+        <v>0.0006970971927042919</v>
       </c>
       <c r="E38" t="n">
         <v>0.000235721612156815</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0003079526746306689</v>
+        <v>0.000307952674630669</v>
       </c>
       <c r="G38" t="n">
-        <v>4.991915880708101e-05</v>
+        <v>4.991915880708104e-05</v>
       </c>
       <c r="H38" t="n">
         <v>3.448684609813101e-05</v>
@@ -2530,7 +2530,7 @@
         <v>1.1656333029178e-05</v>
       </c>
       <c r="M38" t="n">
-        <v>6.69940409574e-06</v>
+        <v>6.699404095739998e-06</v>
       </c>
       <c r="N38" t="n">
         <v>9.28676371628e-07</v>
@@ -2555,10 +2555,10 @@
         <v>0.001929213357103222</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0009394734289056795</v>
+        <v>0.0009394734289056798</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0008402638097944402</v>
+        <v>0.00084026380979444</v>
       </c>
       <c r="E39" t="n">
         <v>0.000214895019258529</v>
@@ -2567,7 +2567,7 @@
         <v>0.000171258717030985</v>
       </c>
       <c r="G39" t="n">
-        <v>5.7835372793224e-05</v>
+        <v>5.783537279322402e-05</v>
       </c>
       <c r="H39" t="n">
         <v>2.602150336141698e-05</v>
@@ -2585,7 +2585,7 @@
         <v>1.0995890906067e-05</v>
       </c>
       <c r="M39" t="n">
-        <v>6.665920496359999e-06</v>
+        <v>6.665920496360001e-06</v>
       </c>
       <c r="N39" t="n">
         <v>8.4109199992e-07</v>
@@ -2610,7 +2610,7 @@
         <v>0.002747249858562731</v>
       </c>
       <c r="C40" t="n">
-        <v>0.001527887137142105</v>
+        <v>0.001527887137142106</v>
       </c>
       <c r="D40" t="n">
         <v>0.001046516732959581</v>
@@ -2619,10 +2619,10 @@
         <v>0.000233633239198027</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0005649980348151131</v>
+        <v>0.000564998034815113</v>
       </c>
       <c r="G40" t="n">
-        <v>8.138702462211699e-05</v>
+        <v>8.138702462211701e-05</v>
       </c>
       <c r="H40" t="n">
         <v>6.645262618887299e-05</v>
@@ -2634,7 +2634,7 @@
         <v>3.885037097167799e-05</v>
       </c>
       <c r="K40" t="n">
-        <v>3.597518816554e-05</v>
+        <v>3.597518816554001e-05</v>
       </c>
       <c r="L40" t="n">
         <v>1.850274511035e-05</v>
@@ -2665,7 +2665,7 @@
         <v>0.002644199476832112</v>
       </c>
       <c r="C41" t="n">
-        <v>0.001396134450982847</v>
+        <v>0.001396134450982848</v>
       </c>
       <c r="D41" t="n">
         <v>0.001069056505015186</v>
@@ -2674,10 +2674,10 @@
         <v>0.000210068926581166</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0004199810356886431</v>
+        <v>0.0004199810356886429</v>
       </c>
       <c r="G41" t="n">
-        <v>7.559166559743299e-05</v>
+        <v>7.559166559743297e-05</v>
       </c>
       <c r="H41" t="n">
         <v>6.509737155465598e-05</v>
@@ -2695,7 +2695,7 @@
         <v>1.5182856845464e-05</v>
       </c>
       <c r="M41" t="n">
-        <v>8.933813097649998e-06</v>
+        <v>8.933813097650002e-06</v>
       </c>
       <c r="N41" t="n">
         <v>1.277958513367e-06</v>
@@ -2729,22 +2729,22 @@
         <v>0.000219025444421981</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0004816518594911269</v>
+        <v>0.000481651859491127</v>
       </c>
       <c r="G42" t="n">
-        <v>8.016834406589399e-05</v>
+        <v>8.0168344065894e-05</v>
       </c>
       <c r="H42" t="n">
         <v>7.250586956475599e-05</v>
       </c>
       <c r="I42" t="n">
-        <v>0.0002218990911244991</v>
+        <v>0.000221899091124499</v>
       </c>
       <c r="J42" t="n">
         <v>3.5851236333572e-05</v>
       </c>
       <c r="K42" t="n">
-        <v>2.983462051458001e-05</v>
+        <v>2.983462051458e-05</v>
       </c>
       <c r="L42" t="n">
         <v>1.5663439923289e-05</v>
@@ -2778,7 +2778,7 @@
         <v>0.001016391622132914</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0009446252311596148</v>
+        <v>0.0009446252311596153</v>
       </c>
       <c r="E43" t="n">
         <v>0.000211861368733999</v>
@@ -2787,7 +2787,7 @@
         <v>0.00016327550200293</v>
       </c>
       <c r="G43" t="n">
-        <v>6.250558847080095e-05</v>
+        <v>6.250558847080096e-05</v>
       </c>
       <c r="H43" t="n">
         <v>2.781322175166601e-05</v>
@@ -2830,10 +2830,10 @@
         <v>0.001692890160240495</v>
       </c>
       <c r="C44" t="n">
-        <v>0.0007880134479967338</v>
+        <v>0.0007880134479967337</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0007110489200537888</v>
+        <v>0.0007110489200537887</v>
       </c>
       <c r="E44" t="n">
         <v>0.000179283497584328</v>
@@ -2842,7 +2842,7 @@
         <v>0.000158589054205992</v>
       </c>
       <c r="G44" t="n">
-        <v>5.214093843198101e-05</v>
+        <v>5.214093843198098e-05</v>
       </c>
       <c r="H44" t="n">
         <v>2.6735553911478e-05</v>
@@ -2860,10 +2860,10 @@
         <v>1.0494296600469e-05</v>
       </c>
       <c r="M44" t="n">
-        <v>6.437938025120001e-06</v>
+        <v>6.43793802512e-06</v>
       </c>
       <c r="N44" t="n">
-        <v>8.273206930549999e-07</v>
+        <v>8.273206930550002e-07</v>
       </c>
       <c r="O44" t="n">
         <v>2.2435953296e-07</v>
@@ -2882,16 +2882,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.001132055144528843</v>
+        <v>0.001132055144528844</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0005936492824849146</v>
+        <v>0.0005936492824849148</v>
       </c>
       <c r="D45" t="n">
-        <v>0.000547014625181137</v>
+        <v>0.0005470146251811371</v>
       </c>
       <c r="E45" t="n">
-        <v>8.120384120442501e-05</v>
+        <v>8.120384120442498e-05</v>
       </c>
       <c r="F45" t="n">
         <v>0.000125710381312225</v>
@@ -2912,7 +2912,7 @@
         <v>1.455237620714e-05</v>
       </c>
       <c r="L45" t="n">
-        <v>6.427842627878001e-06</v>
+        <v>6.427842627878e-06</v>
       </c>
       <c r="M45" t="n">
         <v>4.418022398885e-06</v>
@@ -2937,16 +2937,16 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.001168372555359731</v>
+        <v>0.001168372555359732</v>
       </c>
       <c r="C46" t="n">
-        <v>0.0005970634948660619</v>
+        <v>0.000597063494866062</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0005587983044892318</v>
+        <v>0.0005587983044892321</v>
       </c>
       <c r="E46" t="n">
-        <v>9.077416008383499e-05</v>
+        <v>9.0774160083835e-05</v>
       </c>
       <c r="F46" t="n">
         <v>0.000117126269562505</v>
@@ -2967,13 +2967,13 @@
         <v>1.641070107304e-05</v>
       </c>
       <c r="L46" t="n">
-        <v>6.642580152757001e-06</v>
+        <v>6.642580152756999e-06</v>
       </c>
       <c r="M46" t="n">
         <v>4.572713602386e-06</v>
       </c>
       <c r="N46" t="n">
-        <v>5.721140868590001e-07</v>
+        <v>5.72114086859e-07</v>
       </c>
       <c r="O46" t="n">
         <v>1.49075581693e-07</v>
@@ -2992,19 +2992,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.001575950372277129</v>
+        <v>0.001575950372277131</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0009146027222371428</v>
+        <v>0.0009146027222371431</v>
       </c>
       <c r="D47" t="n">
-        <v>0.00065937744821812</v>
+        <v>0.0006593774482181199</v>
       </c>
       <c r="E47" t="n">
         <v>0.000117136149649273</v>
       </c>
       <c r="F47" t="n">
-        <v>0.000331702296992018</v>
+        <v>0.0003317022969920181</v>
       </c>
       <c r="G47" t="n">
         <v>4.5145592713797e-05</v>
@@ -3025,10 +3025,10 @@
         <v>9.605556304322e-06</v>
       </c>
       <c r="M47" t="n">
-        <v>5.450156439617999e-06</v>
+        <v>5.450156439618e-06</v>
       </c>
       <c r="N47" t="n">
-        <v>5.87657569629e-07</v>
+        <v>5.876575696289999e-07</v>
       </c>
       <c r="O47" t="n">
         <v>1.06245612254e-07</v>
@@ -3047,10 +3047,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.002255374866666666</v>
+        <v>0.002255374866666667</v>
       </c>
       <c r="C48" t="n">
-        <v>0.001266130033333334</v>
+        <v>0.001266130033333333</v>
       </c>
       <c r="D48" t="n">
         <v>0.001037378033333334</v>
@@ -3062,7 +3062,7 @@
         <v>0.0004933461666666667</v>
       </c>
       <c r="G48" t="n">
-        <v>7.797876666666669e-05</v>
+        <v>7.797876666666671e-05</v>
       </c>
       <c r="H48" t="n">
         <v>2.816486666666667e-05</v>
@@ -3074,16 +3074,16 @@
         <v>4.979523333333332e-05</v>
       </c>
       <c r="K48" t="n">
-        <v>7.714166666666665e-05</v>
+        <v>7.714166666666667e-05</v>
       </c>
       <c r="L48" t="n">
-        <v>7.947133333333335e-05</v>
+        <v>7.947133333333333e-05</v>
       </c>
       <c r="M48" t="n">
         <v>1.39649e-05</v>
       </c>
       <c r="N48" t="n">
-        <v>6.848666666666666e-07</v>
+        <v>6.848666666666665e-07</v>
       </c>
       <c r="O48" t="n">
         <v>8.019999999999999e-08</v>
@@ -3100,13 +3100,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.002184562727940543</v>
+        <v>0.002184562727940542</v>
       </c>
       <c r="C49" t="n">
         <v>0.001001353325778946</v>
       </c>
       <c r="D49" t="n">
-        <v>0.0006386694694071304</v>
+        <v>0.0006386694694071306</v>
       </c>
       <c r="E49" t="n">
         <v>0.000240649404328375</v>
@@ -3121,13 +3121,13 @@
         <v>4.069776559558712e-05</v>
       </c>
       <c r="I49" t="n">
-        <v>5.8943292567826e-05</v>
+        <v>5.894329256782601e-05</v>
       </c>
       <c r="J49" t="n">
         <v>5.954881027014721e-05</v>
       </c>
       <c r="K49" t="n">
-        <v>3.172790139976217e-05</v>
+        <v>3.172790139976218e-05</v>
       </c>
       <c r="L49" t="n">
         <v>2.316160207538012e-05</v>
@@ -3136,7 +3136,7 @@
         <v>1.586527368234073e-05</v>
       </c>
       <c r="N49" t="n">
-        <v>2.844998791466065e-06</v>
+        <v>2.844998791466066e-06</v>
       </c>
       <c r="O49" t="n">
         <v>5.372710064720235e-07</v>
@@ -3158,19 +3158,19 @@
         <v>0.002104601662986183</v>
       </c>
       <c r="C50" t="n">
-        <v>0.0009821250070586134</v>
+        <v>0.0009821250070586136</v>
       </c>
       <c r="D50" t="n">
-        <v>0.0005484747843320167</v>
+        <v>0.0005484747843320174</v>
       </c>
       <c r="E50" t="n">
-        <v>0.0002429590163998539</v>
+        <v>0.000242959016399854</v>
       </c>
       <c r="F50" t="n">
-        <v>5.246978427922783e-05</v>
+        <v>5.246978427922782e-05</v>
       </c>
       <c r="G50" t="n">
-        <v>0.0001432473729292475</v>
+        <v>0.0001432473729292474</v>
       </c>
       <c r="H50" t="n">
         <v>3.933039678551726e-05</v>
@@ -3182,7 +3182,7 @@
         <v>6.218338205725706e-05</v>
       </c>
       <c r="K50" t="n">
-        <v>3.802500242506151e-05</v>
+        <v>3.80250024250615e-05</v>
       </c>
       <c r="L50" t="n">
         <v>2.435423076804001e-05</v>
@@ -3191,7 +3191,7 @@
         <v>1.84867749090471e-05</v>
       </c>
       <c r="N50" t="n">
-        <v>3.238349699934597e-06</v>
+        <v>3.238349699934596e-06</v>
       </c>
       <c r="O50" t="n">
         <v>6.120538746817381e-07</v>
@@ -3216,7 +3216,7 @@
         <v>0.001385092464708465</v>
       </c>
       <c r="D51" t="n">
-        <v>0.0006933205638113998</v>
+        <v>0.0006933205638113997</v>
       </c>
       <c r="E51" t="n">
         <v>0.0003245908282213207</v>
@@ -3237,7 +3237,7 @@
         <v>8.040793548814298e-05</v>
       </c>
       <c r="K51" t="n">
-        <v>3.510689864461558e-05</v>
+        <v>3.510689864461559e-05</v>
       </c>
       <c r="L51" t="n">
         <v>2.330639946019494e-05</v>
@@ -3246,7 +3246,7 @@
         <v>1.503870544899254e-05</v>
       </c>
       <c r="N51" t="n">
-        <v>2.999832958646122e-06</v>
+        <v>2.999832958646123e-06</v>
       </c>
       <c r="O51" t="n">
         <v>6.666624439283216e-07</v>
@@ -3271,10 +3271,10 @@
         <v>0.001331765041888567</v>
       </c>
       <c r="D52" t="n">
-        <v>0.0006155648967384228</v>
+        <v>0.0006155648967384225</v>
       </c>
       <c r="E52" t="n">
-        <v>0.0003211560737995639</v>
+        <v>0.0003211560737995638</v>
       </c>
       <c r="F52" t="n">
         <v>0.0001037806284532741</v>
@@ -3295,7 +3295,7 @@
         <v>3.740574487800726e-05</v>
       </c>
       <c r="L52" t="n">
-        <v>1.931379165727816e-05</v>
+        <v>1.931379165727817e-05</v>
       </c>
       <c r="M52" t="n">
         <v>1.577233402933301e-05</v>
@@ -3320,7 +3320,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.004632372349213295</v>
+        <v>0.004632372349213293</v>
       </c>
       <c r="C53" t="n">
         <v>0.00251244407127723</v>
@@ -3335,7 +3335,7 @@
         <v>0.0005760074691448202</v>
       </c>
       <c r="G53" t="n">
-        <v>0.0001731978164102897</v>
+        <v>0.0001731978164102896</v>
       </c>
       <c r="H53" t="n">
         <v>8.948261675993123e-05</v>
@@ -3375,28 +3375,28 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.002668216445547569</v>
+        <v>0.002668216445547567</v>
       </c>
       <c r="C54" t="n">
         <v>0.001745718676149256</v>
       </c>
       <c r="D54" t="n">
-        <v>0.001217356698369616</v>
+        <v>0.001217356698369617</v>
       </c>
       <c r="E54" t="n">
-        <v>0.0003473150048107284</v>
+        <v>0.0003473150048107285</v>
       </c>
       <c r="F54" t="n">
-        <v>0.000415960962413723</v>
+        <v>0.0004159609624137231</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0001472291493376383</v>
+        <v>0.0001472291493376382</v>
       </c>
       <c r="H54" t="n">
         <v>2.935898471152523e-05</v>
       </c>
       <c r="I54" t="n">
-        <v>9.939429550818977e-06</v>
+        <v>9.939429550818979e-06</v>
       </c>
       <c r="J54" t="n">
         <v>7.602498357553645e-05</v>
@@ -3411,7 +3411,7 @@
         <v>2.016953955373296e-05</v>
       </c>
       <c r="N54" t="n">
-        <v>3.298424832014455e-06</v>
+        <v>3.298424832014456e-06</v>
       </c>
       <c r="O54" t="n">
         <v>5.05192606840639e-07</v>
@@ -3430,19 +3430,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.004593450969256783</v>
+        <v>0.004593450969256785</v>
       </c>
       <c r="C55" t="n">
-        <v>0.002698702211308841</v>
+        <v>0.002698702211308842</v>
       </c>
       <c r="D55" t="n">
-        <v>0.001800835855612344</v>
+        <v>0.001800835855612345</v>
       </c>
       <c r="E55" t="n">
         <v>0.0005015693095362459</v>
       </c>
       <c r="F55" t="n">
-        <v>0.0006626988762114163</v>
+        <v>0.0006626988762114164</v>
       </c>
       <c r="G55" t="n">
         <v>0.0002364314851198428</v>
@@ -3457,10 +3457,10 @@
         <v>9.355486789842817e-05</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0001471686852333628</v>
+        <v>0.0001471686852333627</v>
       </c>
       <c r="L55" t="n">
-        <v>8.409606758615346e-05</v>
+        <v>8.409606758615347e-05</v>
       </c>
       <c r="M55" t="n">
         <v>2.541533408864252e-05</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.002101101616301523</v>
+        <v>0.002101101616301526</v>
       </c>
       <c r="C56" t="n">
         <v>0.00145207657031868</v>
@@ -3500,25 +3500,25 @@
         <v>0.0003338121150566797</v>
       </c>
       <c r="G56" t="n">
-        <v>0.0001192015273042979</v>
+        <v>0.0001192015273042978</v>
       </c>
       <c r="H56" t="n">
         <v>2.329169796938328e-05</v>
       </c>
       <c r="I56" t="n">
-        <v>9.831451816116536e-06</v>
+        <v>9.831451816116538e-06</v>
       </c>
       <c r="J56" t="n">
         <v>6.657085042573176e-05</v>
       </c>
       <c r="K56" t="n">
-        <v>6.680362340021648e-05</v>
+        <v>6.680362340021646e-05</v>
       </c>
       <c r="L56" t="n">
-        <v>3.869193351669941e-05</v>
+        <v>3.869193351669942e-05</v>
       </c>
       <c r="M56" t="n">
-        <v>1.699732864298232e-05</v>
+        <v>1.699732864298233e-05</v>
       </c>
       <c r="N56" t="n">
         <v>2.5175342124117e-06</v>
@@ -3540,10 +3540,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.002644052098955674</v>
+        <v>0.002644052098955676</v>
       </c>
       <c r="C57" t="n">
-        <v>0.001482720423119658</v>
+        <v>0.001482720423119657</v>
       </c>
       <c r="D57" t="n">
         <v>0.001083894990472623</v>
@@ -3552,10 +3552,10 @@
         <v>0.000267153326006525</v>
       </c>
       <c r="F57" t="n">
-        <v>0.0003090901511531718</v>
+        <v>0.0003090901511531719</v>
       </c>
       <c r="G57" t="n">
-        <v>8.485516322868907e-05</v>
+        <v>8.485516322868904e-05</v>
       </c>
       <c r="H57" t="n">
         <v>2.093391656660262e-05</v>
@@ -3567,7 +3567,7 @@
         <v>5.352354042131278e-05</v>
       </c>
       <c r="K57" t="n">
-        <v>5.881637728487493e-05</v>
+        <v>5.881637728487495e-05</v>
       </c>
       <c r="L57" t="n">
         <v>3.590733664153508e-05</v>
@@ -3607,7 +3607,7 @@
         <v>0.0002658898361476365</v>
       </c>
       <c r="F58" t="n">
-        <v>0.00029954387749905</v>
+        <v>0.0002995438774990501</v>
       </c>
       <c r="G58" t="n">
         <v>8.04906032079881e-05</v>
@@ -3622,7 +3622,7 @@
         <v>5.308895429508855e-05</v>
       </c>
       <c r="K58" t="n">
-        <v>5.67871597862308e-05</v>
+        <v>5.678715978623079e-05</v>
       </c>
       <c r="L58" t="n">
         <v>3.442182996505496e-05</v>
@@ -3648,22 +3648,22 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.002835660686174028</v>
+        <v>0.002835660686174027</v>
       </c>
       <c r="C59" t="n">
-        <v>0.00155160058903696</v>
+        <v>0.001551600589036959</v>
       </c>
       <c r="D59" t="n">
-        <v>0.001103382733073639</v>
+        <v>0.00110338273307364</v>
       </c>
       <c r="E59" t="n">
-        <v>0.0002602720531031089</v>
+        <v>0.000260272053103109</v>
       </c>
       <c r="F59" t="n">
-        <v>0.0003274334497234606</v>
+        <v>0.0003274334497234605</v>
       </c>
       <c r="G59" t="n">
-        <v>9.615315778171082e-05</v>
+        <v>9.615315778171085e-05</v>
       </c>
       <c r="H59" t="n">
         <v>1.714202430046671e-05</v>
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.002706242834833999</v>
+        <v>0.002706242834834002</v>
       </c>
       <c r="C60" t="n">
         <v>0.001494748973052823</v>
@@ -3712,13 +3712,13 @@
         <v>0.001073739604374053</v>
       </c>
       <c r="E60" t="n">
-        <v>0.0002632887824461379</v>
+        <v>0.000263288782446138</v>
       </c>
       <c r="F60" t="n">
         <v>0.0003169689169855</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0001043961775919132</v>
+        <v>0.0001043961775919133</v>
       </c>
       <c r="H60" t="n">
         <v>2.692123522126264e-05</v>
@@ -3733,7 +3733,7 @@
         <v>6.552864969507031e-05</v>
       </c>
       <c r="L60" t="n">
-        <v>3.703729366398552e-05</v>
+        <v>3.703729366398553e-05</v>
       </c>
       <c r="M60" t="n">
         <v>1.572624615614269e-05</v>
@@ -3758,7 +3758,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.003747387877857536</v>
+        <v>0.003747387877857538</v>
       </c>
       <c r="C61" t="n">
         <v>0.00169004397275377</v>
@@ -3770,7 +3770,7 @@
         <v>0.0002227113274684656</v>
       </c>
       <c r="F61" t="n">
-        <v>0.0003264617926132513</v>
+        <v>0.0003264617926132514</v>
       </c>
       <c r="G61" t="n">
         <v>0.0001510864194647791</v>
@@ -3788,7 +3788,7 @@
         <v>0.000117221845859349</v>
       </c>
       <c r="L61" t="n">
-        <v>6.96368276046164e-05</v>
+        <v>6.963682760461641e-05</v>
       </c>
       <c r="M61" t="n">
         <v>4.918241245971438e-05</v>
@@ -3811,13 +3811,13 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.003706208915424827</v>
+        <v>0.003706208915424828</v>
       </c>
       <c r="C62" t="n">
         <v>0.001545779362900664</v>
       </c>
       <c r="D62" t="n">
-        <v>0.001191488952461691</v>
+        <v>0.00119148895246169</v>
       </c>
       <c r="E62" t="n">
         <v>0.0001149206766298572</v>
@@ -3867,7 +3867,7 @@
         <v>0.003686241299394129</v>
       </c>
       <c r="C63" t="n">
-        <v>0.001380702166290202</v>
+        <v>0.001380702166290203</v>
       </c>
       <c r="D63" t="n">
         <v>0.00101091353507074</v>
@@ -3891,13 +3891,13 @@
         <v>8.818509571645631e-05</v>
       </c>
       <c r="K63" t="n">
-        <v>9.153488074513452e-05</v>
+        <v>9.153488074513451e-05</v>
       </c>
       <c r="L63" t="n">
-        <v>6.156126215509797e-05</v>
+        <v>6.156126215509798e-05</v>
       </c>
       <c r="M63" t="n">
-        <v>5.106621016589174e-06</v>
+        <v>5.106621016589173e-06</v>
       </c>
       <c r="N63" t="n">
         <v>1.004285235137828e-06</v>
@@ -3944,10 +3944,10 @@
         <v>9.184817507794753e-05</v>
       </c>
       <c r="K64" t="n">
-        <v>7.847773906469612e-05</v>
+        <v>7.847773906469611e-05</v>
       </c>
       <c r="L64" t="n">
-        <v>4.938944684008635e-05</v>
+        <v>4.938944684008636e-05</v>
       </c>
       <c r="M64" t="n">
         <v>7.956760738641646e-06</v>
@@ -3970,7 +3970,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.004033248271664659</v>
+        <v>0.004033248271664658</v>
       </c>
       <c r="C65" t="n">
         <v>0.001808862512918449</v>
@@ -4000,13 +4000,13 @@
         <v>0.000125393364241531</v>
       </c>
       <c r="L65" t="n">
-        <v>7.36134269103288e-05</v>
+        <v>7.361342691032879e-05</v>
       </c>
       <c r="M65" t="n">
-        <v>4.832644064174692e-05</v>
+        <v>4.832644064174693e-05</v>
       </c>
       <c r="N65" t="n">
-        <v>2.720649865327134e-06</v>
+        <v>2.720649865327133e-06</v>
       </c>
       <c r="O65" t="n">
         <v>2.981769179674527e-07</v>
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.004040923374042935</v>
+        <v>0.004040923374042934</v>
       </c>
       <c r="C66" t="n">
         <v>0.001851308025002989</v>
@@ -4032,10 +4032,10 @@
         <v>0.001318184803202773</v>
       </c>
       <c r="E66" t="n">
-        <v>0.0002280502256120225</v>
+        <v>0.0002280502256120226</v>
       </c>
       <c r="F66" t="n">
-        <v>0.000335170017905181</v>
+        <v>0.0003351700179051811</v>
       </c>
       <c r="G66" t="n">
         <v>0.0001490913279728661</v>
@@ -4076,10 +4076,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.004288052833700116</v>
+        <v>0.004288052833700113</v>
       </c>
       <c r="C67" t="n">
-        <v>0.001923197859947143</v>
+        <v>0.001923197859947144</v>
       </c>
       <c r="D67" t="n">
         <v>0.001370477475251594</v>
@@ -4088,7 +4088,7 @@
         <v>0.0001988387227540186</v>
       </c>
       <c r="F67" t="n">
-        <v>0.0003212751597537197</v>
+        <v>0.0003212751597537196</v>
       </c>
       <c r="G67" t="n">
         <v>0.000140841488228097</v>
@@ -4129,13 +4129,13 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.003909022933193027</v>
+        <v>0.003909022933193026</v>
       </c>
       <c r="C68" t="n">
-        <v>0.001787588763581899</v>
+        <v>0.0017875887635819</v>
       </c>
       <c r="D68" t="n">
-        <v>0.001288753332503702</v>
+        <v>0.001288753332503703</v>
       </c>
       <c r="E68" t="n">
         <v>0.0002712925932323812</v>
@@ -4159,10 +4159,10 @@
         <v>0.0001022576210222351</v>
       </c>
       <c r="L68" t="n">
-        <v>7.480174031418134e-05</v>
+        <v>7.480174031418133e-05</v>
       </c>
       <c r="M68" t="n">
-        <v>2.332135252261706e-05</v>
+        <v>2.332135252261707e-05</v>
       </c>
       <c r="N68" t="n">
         <v>7.965687019262703e-07</v>
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.003745110287647575</v>
+        <v>0.003745110287647577</v>
       </c>
       <c r="C69" t="n">
         <v>0.00165906310731707</v>
@@ -4235,13 +4235,13 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.003049252700574094</v>
+        <v>0.003049252700574093</v>
       </c>
       <c r="C70" t="n">
         <v>0.001744132325382065</v>
       </c>
       <c r="D70" t="n">
-        <v>0.001334581157779442</v>
+        <v>0.001334581157779441</v>
       </c>
       <c r="E70" t="n">
         <v>0.0002795085552511624</v>
@@ -4265,7 +4265,7 @@
         <v>7.115565376222185e-05</v>
       </c>
       <c r="L70" t="n">
-        <v>5.792985773580206e-05</v>
+        <v>5.792985773580205e-05</v>
       </c>
       <c r="M70" t="n">
         <v>1.589107871683826e-05</v>
@@ -4288,22 +4288,22 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.004293678498550643</v>
+        <v>0.004293678498550642</v>
       </c>
       <c r="C71" t="n">
         <v>0.001325237585336988</v>
       </c>
       <c r="D71" t="n">
-        <v>0.0006765593457452466</v>
+        <v>0.000676559345745247</v>
       </c>
       <c r="E71" t="n">
-        <v>0.0001584466283220529</v>
+        <v>0.0001584466283220528</v>
       </c>
       <c r="F71" t="n">
-        <v>8.082248280696802e-05</v>
+        <v>8.0822482806968e-05</v>
       </c>
       <c r="G71" t="n">
-        <v>0.0001208878676820726</v>
+        <v>0.0001208878676820725</v>
       </c>
       <c r="H71" t="n">
         <v>1.92781319723612e-05</v>
@@ -4315,7 +4315,7 @@
         <v>0.0001169349607233861</v>
       </c>
       <c r="K71" t="n">
-        <v>8.552688730680397e-05</v>
+        <v>8.552688730680395e-05</v>
       </c>
       <c r="L71" t="n">
         <v>0.0001681088945226711</v>
@@ -4343,28 +4343,28 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.004631520566891492</v>
+        <v>0.004631520566891494</v>
       </c>
       <c r="C72" t="n">
-        <v>0.001358688626539661</v>
+        <v>0.00135868862653966</v>
       </c>
       <c r="D72" t="n">
-        <v>0.0006730639148965215</v>
+        <v>0.0006730639148965214</v>
       </c>
       <c r="E72" t="n">
         <v>8.59136206728588e-05</v>
       </c>
       <c r="F72" t="n">
-        <v>6.374019454646459e-05</v>
+        <v>6.374019454646457e-05</v>
       </c>
       <c r="G72" t="n">
-        <v>0.0001516138959986469</v>
+        <v>0.000151613895998647</v>
       </c>
       <c r="H72" t="n">
         <v>2.925622753909315e-05</v>
       </c>
       <c r="I72" t="n">
-        <v>0.0002998740530377892</v>
+        <v>0.0002998740530377891</v>
       </c>
       <c r="J72" t="n">
         <v>0.0001373235967779671</v>
@@ -4398,7 +4398,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.002252902970923498</v>
+        <v>0.002252902970923499</v>
       </c>
       <c r="C73" t="n">
         <v>0.001043392762746281</v>
@@ -4410,22 +4410,22 @@
         <v>0.0002391356896909046</v>
       </c>
       <c r="F73" t="n">
-        <v>5.765261136181501e-05</v>
+        <v>5.7652611361815e-05</v>
       </c>
       <c r="G73" t="n">
-        <v>0.0001545350947195124</v>
+        <v>0.0001545350947195125</v>
       </c>
       <c r="H73" t="n">
         <v>4.218095884751349e-05</v>
       </c>
       <c r="I73" t="n">
-        <v>6.80177315902709e-05</v>
+        <v>6.801773159027093e-05</v>
       </c>
       <c r="J73" t="n">
         <v>6.045936783044685e-05</v>
       </c>
       <c r="K73" t="n">
-        <v>3.999438828429678e-05</v>
+        <v>3.999438828429679e-05</v>
       </c>
       <c r="L73" t="n">
         <v>2.752284242561429e-05</v>
@@ -4453,22 +4453,22 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.002166721066990613</v>
+        <v>0.002166721066990611</v>
       </c>
       <c r="C74" t="n">
-        <v>0.0009050305949668675</v>
+        <v>0.0009050305949668678</v>
       </c>
       <c r="D74" t="n">
-        <v>0.0005628174997770615</v>
+        <v>0.0005628174997770618</v>
       </c>
       <c r="E74" t="n">
         <v>0.0002133779050954858</v>
       </c>
       <c r="F74" t="n">
-        <v>5.473294454966051e-05</v>
+        <v>5.47329445496605e-05</v>
       </c>
       <c r="G74" t="n">
-        <v>0.0001284854737524962</v>
+        <v>0.0001284854737524963</v>
       </c>
       <c r="H74" t="n">
         <v>5.016332377030962e-05</v>
@@ -4489,7 +4489,7 @@
         <v>1.942860664872286e-05</v>
       </c>
       <c r="N74" t="n">
-        <v>3.048208144374993e-06</v>
+        <v>3.048208144374992e-06</v>
       </c>
       <c r="O74" t="n">
         <v>5.752489422288217e-07</v>
@@ -4508,7 +4508,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.004336498143661241</v>
+        <v>0.004336498143661243</v>
       </c>
       <c r="C75" t="n">
         <v>0.001239974648819916</v>
@@ -4538,7 +4538,7 @@
         <v>9.155687496592259e-05</v>
       </c>
       <c r="L75" t="n">
-        <v>0.0002511236843627302</v>
+        <v>0.0002511236843627303</v>
       </c>
       <c r="M75" t="n">
         <v>2.389712259759261e-05</v>
@@ -4569,13 +4569,13 @@
         <v>0.001222347340293859</v>
       </c>
       <c r="D76" t="n">
-        <v>0.0006382714511713476</v>
+        <v>0.0006382714511713473</v>
       </c>
       <c r="E76" t="n">
-        <v>0.000100301203158066</v>
+        <v>0.0001003012031580659</v>
       </c>
       <c r="F76" t="n">
-        <v>6.548925849639757e-05</v>
+        <v>6.548925849639756e-05</v>
       </c>
       <c r="G76" t="n">
         <v>0.000132959754693479</v>
@@ -4584,13 +4584,13 @@
         <v>2.3826886357102e-05</v>
       </c>
       <c r="I76" t="n">
-        <v>0.0002728483846868518</v>
+        <v>0.0002728483846868517</v>
       </c>
       <c r="J76" t="n">
         <v>0.0001141898159997968</v>
       </c>
       <c r="K76" t="n">
-        <v>8.284786674625626e-05</v>
+        <v>8.284786674625627e-05</v>
       </c>
       <c r="L76" t="n">
         <v>0.0002083909380165502</v>
@@ -4599,7 +4599,7 @@
         <v>1.938609134808886e-05</v>
       </c>
       <c r="N76" t="n">
-        <v>2.303899681316164e-06</v>
+        <v>2.303899681316165e-06</v>
       </c>
       <c r="O76" t="n">
         <v>7.199368199366079e-07</v>
@@ -4618,16 +4618,16 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.005959005379741445</v>
+        <v>0.005959005379741454</v>
       </c>
       <c r="C77" t="n">
-        <v>0.001466803960294855</v>
+        <v>0.001466803960294854</v>
       </c>
       <c r="D77" t="n">
-        <v>0.0005391263945216694</v>
+        <v>0.0005391263945216695</v>
       </c>
       <c r="E77" t="n">
-        <v>8.895662473699249e-05</v>
+        <v>8.895662473699246e-05</v>
       </c>
       <c r="F77" t="n">
         <v>4.755022936279851e-05</v>
@@ -4645,7 +4645,7 @@
         <v>0.0001636388651370349</v>
       </c>
       <c r="K77" t="n">
-        <v>9.744477117491422e-05</v>
+        <v>9.744477117491421e-05</v>
       </c>
       <c r="L77" t="n">
         <v>0.000386822364174485</v>
@@ -4654,7 +4654,7 @@
         <v>2.178671155777837e-05</v>
       </c>
       <c r="N77" t="n">
-        <v>2.079784171227332e-06</v>
+        <v>2.079784171227331e-06</v>
       </c>
       <c r="O77" t="n">
         <v>6.221736829115317e-07</v>
@@ -4673,19 +4673,19 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.00455847125931526</v>
+        <v>0.004558471259315262</v>
       </c>
       <c r="C78" t="n">
-        <v>0.001285088599691144</v>
+        <v>0.001285088599691145</v>
       </c>
       <c r="D78" t="n">
-        <v>0.0006923160968336961</v>
+        <v>0.0006923160968336963</v>
       </c>
       <c r="E78" t="n">
         <v>0.0001138909618399733</v>
       </c>
       <c r="F78" t="n">
-        <v>6.677200924643892e-05</v>
+        <v>6.677200924643893e-05</v>
       </c>
       <c r="G78" t="n">
         <v>0.0001988491257506812</v>
@@ -4694,16 +4694,16 @@
         <v>3.038435926426904e-05</v>
       </c>
       <c r="I78" t="n">
-        <v>0.0003321944326705517</v>
+        <v>0.0003321944326705518</v>
       </c>
       <c r="J78" t="n">
         <v>0.0001092632438432839</v>
       </c>
       <c r="K78" t="n">
-        <v>8.106118729614012e-05</v>
+        <v>8.106118729614013e-05</v>
       </c>
       <c r="L78" t="n">
-        <v>0.0002256711643254289</v>
+        <v>0.000225671164325429</v>
       </c>
       <c r="M78" t="n">
         <v>2.10784737322434e-05</v>
@@ -4728,13 +4728,13 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.004664884701021463</v>
+        <v>0.004664884701021462</v>
       </c>
       <c r="C79" t="n">
-        <v>0.001014875754617674</v>
+        <v>0.001014875754617675</v>
       </c>
       <c r="D79" t="n">
-        <v>0.0006144408527671524</v>
+        <v>0.000614440852767153</v>
       </c>
       <c r="E79" t="n">
         <v>9.596766635880299e-05</v>
@@ -4743,13 +4743,13 @@
         <v>6.784134826347187e-05</v>
       </c>
       <c r="G79" t="n">
-        <v>0.0001719012980263556</v>
+        <v>0.0001719012980263557</v>
       </c>
       <c r="H79" t="n">
         <v>3.37341347654996e-05</v>
       </c>
       <c r="I79" t="n">
-        <v>0.0002896018560624719</v>
+        <v>0.0002896018560624718</v>
       </c>
       <c r="J79" t="n">
         <v>0.0001311267771574311</v>
@@ -4758,7 +4758,7 @@
         <v>9.182252970823659e-05</v>
       </c>
       <c r="L79" t="n">
-        <v>0.000122130475182102</v>
+        <v>0.0001221304751821021</v>
       </c>
       <c r="M79" t="n">
         <v>2.064856471705259e-05</v>
@@ -4783,19 +4783,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.00206976235135736</v>
+        <v>0.002069762351357361</v>
       </c>
       <c r="C80" t="n">
-        <v>0.0006775268145180985</v>
+        <v>0.0006775268145180982</v>
       </c>
       <c r="D80" t="n">
-        <v>0.0005221502033828371</v>
+        <v>0.0005221502033828372</v>
       </c>
       <c r="E80" t="n">
         <v>0.0001292410559748941</v>
       </c>
       <c r="F80" t="n">
-        <v>4.447840439255906e-05</v>
+        <v>4.447840439255905e-05</v>
       </c>
       <c r="G80" t="n">
         <v>0.0001910584577852782</v>
@@ -4810,7 +4810,7 @@
         <v>4.565119882872989e-05</v>
       </c>
       <c r="K80" t="n">
-        <v>3.380092889672296e-05</v>
+        <v>3.380092889672297e-05</v>
       </c>
       <c r="L80" t="n">
         <v>1.200068915125211e-05</v>
@@ -4838,10 +4838,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.002720839204821043</v>
+        <v>0.002720839204821042</v>
       </c>
       <c r="C81" t="n">
-        <v>0.0007305625668306809</v>
+        <v>0.0007305625668306808</v>
       </c>
       <c r="D81" t="n">
         <v>0.0004798122103503246</v>
@@ -4853,7 +4853,7 @@
         <v>4.231031597907948e-05</v>
       </c>
       <c r="G81" t="n">
-        <v>0.0001924804796990976</v>
+        <v>0.0001924804796990977</v>
       </c>
       <c r="H81" t="n">
         <v>3.913944197120943e-05</v>
@@ -4865,7 +4865,7 @@
         <v>5.373828753486789e-05</v>
       </c>
       <c r="K81" t="n">
-        <v>4.719106504600213e-05</v>
+        <v>4.719106504600212e-05</v>
       </c>
       <c r="L81" t="n">
         <v>1.803243699840493e-05</v>
@@ -4893,13 +4893,13 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.002454215271207162</v>
+        <v>0.002454215271207165</v>
       </c>
       <c r="C82" t="n">
         <v>0.001365941646129984</v>
       </c>
       <c r="D82" t="n">
-        <v>0.0008293148446994606</v>
+        <v>0.0008293148446994602</v>
       </c>
       <c r="E82" t="n">
         <v>0.0002571076266247518</v>
@@ -4920,10 +4920,10 @@
         <v>3.591548563734665e-05</v>
       </c>
       <c r="K82" t="n">
-        <v>7.839612498854157e-05</v>
+        <v>7.839612498854154e-05</v>
       </c>
       <c r="L82" t="n">
-        <v>5.944792152390173e-05</v>
+        <v>5.944792152390172e-05</v>
       </c>
       <c r="M82" t="n">
         <v>1.504187770531209e-05</v>
@@ -4946,16 +4946,16 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.00258813050447753</v>
+        <v>0.002588130504477531</v>
       </c>
       <c r="C83" t="n">
         <v>0.001419685377689362</v>
       </c>
       <c r="D83" t="n">
-        <v>0.0008432426361361013</v>
+        <v>0.0008432426361361005</v>
       </c>
       <c r="E83" t="n">
-        <v>0.0002640348066557464</v>
+        <v>0.0002640348066557465</v>
       </c>
       <c r="F83" t="n">
         <v>0.0003463165772779967</v>
@@ -4973,10 +4973,10 @@
         <v>3.745330409143174e-05</v>
       </c>
       <c r="K83" t="n">
-        <v>8.63779996644289e-05</v>
+        <v>8.637799966442892e-05</v>
       </c>
       <c r="L83" t="n">
-        <v>6.052421993735147e-05</v>
+        <v>6.052421993735148e-05</v>
       </c>
       <c r="M83" t="n">
         <v>1.620859005056548e-05</v>
@@ -5002,16 +5002,16 @@
         <v>0.002668354227325503</v>
       </c>
       <c r="C84" t="n">
-        <v>0.001331394541248587</v>
+        <v>0.001331394541248586</v>
       </c>
       <c r="D84" t="n">
-        <v>0.0008712655821684414</v>
+        <v>0.0008712655821684409</v>
       </c>
       <c r="E84" t="n">
         <v>0.000220537726473756</v>
       </c>
       <c r="F84" t="n">
-        <v>0.0003047627129898815</v>
+        <v>0.0003047627129898814</v>
       </c>
       <c r="G84" t="n">
         <v>0.0001352218832981502</v>
@@ -5020,7 +5020,7 @@
         <v>3.908973832921965e-05</v>
       </c>
       <c r="I84" t="n">
-        <v>5.947664014193207e-05</v>
+        <v>5.947664014193208e-05</v>
       </c>
       <c r="J84" t="n">
         <v>4.511613582821256e-05</v>
@@ -5035,7 +5035,7 @@
         <v>1.653315746078687e-05</v>
       </c>
       <c r="N84" t="n">
-        <v>1.807899057132292e-06</v>
+        <v>1.807899057132291e-06</v>
       </c>
       <c r="O84" t="n">
         <v>2.867172943282357e-07</v>
@@ -5052,22 +5052,22 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.002850408685037662</v>
+        <v>0.002850408685037661</v>
       </c>
       <c r="C85" t="n">
         <v>0.001345221618198644</v>
       </c>
       <c r="D85" t="n">
-        <v>0.0009192620887719067</v>
+        <v>0.0009192620887719065</v>
       </c>
       <c r="E85" t="n">
         <v>0.0002023960354386911</v>
       </c>
       <c r="F85" t="n">
-        <v>0.0002874233779499023</v>
+        <v>0.0002874233779499024</v>
       </c>
       <c r="G85" t="n">
-        <v>0.0001442194152377239</v>
+        <v>0.0001442194152377238</v>
       </c>
       <c r="H85" t="n">
         <v>3.888402875660148e-05</v>
@@ -5082,7 +5082,7 @@
         <v>0.0001121229865885275</v>
       </c>
       <c r="L85" t="n">
-        <v>5.687055763370441e-05</v>
+        <v>5.687055763370442e-05</v>
       </c>
       <c r="M85" t="n">
         <v>1.669734359253458e-05</v>
@@ -5105,28 +5105,28 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.002053846843991832</v>
+        <v>0.002053846843991833</v>
       </c>
       <c r="C86" t="n">
         <v>0.0008715781793176729</v>
       </c>
       <c r="D86" t="n">
-        <v>0.0006511341803808787</v>
+        <v>0.0006511341803808789</v>
       </c>
       <c r="E86" t="n">
-        <v>0.0001077698193660481</v>
+        <v>0.000107769819366048</v>
       </c>
       <c r="F86" t="n">
         <v>0.0001666499839013095</v>
       </c>
       <c r="G86" t="n">
-        <v>9.78640584452453e-05</v>
+        <v>9.786405844524528e-05</v>
       </c>
       <c r="H86" t="n">
         <v>2.586675425255619e-05</v>
       </c>
       <c r="I86" t="n">
-        <v>5.321869670610356e-05</v>
+        <v>5.321869670610355e-05</v>
       </c>
       <c r="J86" t="n">
         <v>3.988680840022982e-05</v>
@@ -5158,13 +5158,13 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.002333210620826676</v>
+        <v>0.002333210620826675</v>
       </c>
       <c r="C87" t="n">
-        <v>0.0009405393536939192</v>
+        <v>0.0009405393536939189</v>
       </c>
       <c r="D87" t="n">
-        <v>0.000722365657594327</v>
+        <v>0.0007223656575943271</v>
       </c>
       <c r="E87" t="n">
         <v>0.0001121537614509555</v>
@@ -5173,7 +5173,7 @@
         <v>0.000166332389313785</v>
       </c>
       <c r="G87" t="n">
-        <v>9.543663114407575e-05</v>
+        <v>9.543663114407576e-05</v>
       </c>
       <c r="H87" t="n">
         <v>2.46019146628846e-05</v>
@@ -5185,10 +5185,10 @@
         <v>4.667091630111133e-05</v>
       </c>
       <c r="K87" t="n">
-        <v>8.200493387474037e-05</v>
+        <v>8.200493387474038e-05</v>
       </c>
       <c r="L87" t="n">
-        <v>3.861097830247286e-05</v>
+        <v>3.861097830247287e-05</v>
       </c>
       <c r="M87" t="n">
         <v>1.159069511315939e-05</v>
@@ -5211,19 +5211,19 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.002384081749479943</v>
+        <v>0.002384081749479945</v>
       </c>
       <c r="C88" t="n">
         <v>0.001001939286291494</v>
       </c>
       <c r="D88" t="n">
-        <v>0.000759040763998469</v>
+        <v>0.0007590407639984688</v>
       </c>
       <c r="E88" t="n">
         <v>0.0001218065519809573</v>
       </c>
       <c r="F88" t="n">
-        <v>0.0001712461393798544</v>
+        <v>0.0001712461393798545</v>
       </c>
       <c r="G88" t="n">
         <v>8.100626714859634e-05</v>
@@ -5264,13 +5264,13 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.00224875342068901</v>
+        <v>0.002248753420689009</v>
       </c>
       <c r="C89" t="n">
-        <v>0.0009912433791582327</v>
+        <v>0.000991243379158233</v>
       </c>
       <c r="D89" t="n">
-        <v>0.0007761112620528266</v>
+        <v>0.0007761112620528263</v>
       </c>
       <c r="E89" t="n">
         <v>0.0001346873590160968</v>
@@ -5294,7 +5294,7 @@
         <v>5.612901330316652e-05</v>
       </c>
       <c r="L89" t="n">
-        <v>2.865507168694977e-05</v>
+        <v>2.865507168694978e-05</v>
       </c>
       <c r="M89" t="n">
         <v>1.133025772298763e-05</v>
@@ -5323,7 +5323,7 @@
         <v>0.0008908031579456471</v>
       </c>
       <c r="D90" t="n">
-        <v>0.0007116335261458146</v>
+        <v>0.000711633526145815</v>
       </c>
       <c r="E90" t="n">
         <v>0.0001327656740373265</v>
@@ -5344,13 +5344,13 @@
         <v>4.754252919383134e-05</v>
       </c>
       <c r="K90" t="n">
-        <v>4.510434022820878e-05</v>
+        <v>4.510434022820877e-05</v>
       </c>
       <c r="L90" t="n">
-        <v>2.148068401562849e-05</v>
+        <v>2.14806840156285e-05</v>
       </c>
       <c r="M90" t="n">
-        <v>9.69922508443259e-06</v>
+        <v>9.699225084432588e-06</v>
       </c>
       <c r="N90" t="n">
         <v>1.573310360490169e-06</v>
@@ -5370,13 +5370,13 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.00121005688272612</v>
+        <v>0.001210056882726121</v>
       </c>
       <c r="C91" t="n">
-        <v>0.0009626144010869094</v>
+        <v>0.0009626144010869097</v>
       </c>
       <c r="D91" t="n">
-        <v>0.0005539041348841125</v>
+        <v>0.0005539041348841126</v>
       </c>
       <c r="E91" t="n">
         <v>0.0002667975575229067</v>
@@ -5391,7 +5391,7 @@
         <v>1.381492916327907e-05</v>
       </c>
       <c r="I91" t="n">
-        <v>8.845484082018466e-06</v>
+        <v>8.845484082018464e-06</v>
       </c>
       <c r="J91" t="n">
         <v>2.110616443297007e-05</v>
@@ -5406,7 +5406,7 @@
         <v>2.481315228216065e-06</v>
       </c>
       <c r="N91" t="n">
-        <v>4.668438579194348e-07</v>
+        <v>4.668438579194347e-07</v>
       </c>
       <c r="O91" t="n">
         <v>9.378370624389937e-08</v>
@@ -5431,7 +5431,7 @@
         <v>0.000989348134262704</v>
       </c>
       <c r="D92" t="n">
-        <v>0.0005780620128966049</v>
+        <v>0.0005780620128966047</v>
       </c>
       <c r="E92" t="n">
         <v>0.0002726712085343925</v>
@@ -5440,13 +5440,13 @@
         <v>0.0002008110453756718</v>
       </c>
       <c r="G92" t="n">
-        <v>2.714407325699149e-05</v>
+        <v>2.714407325699148e-05</v>
       </c>
       <c r="H92" t="n">
         <v>1.202251321779824e-05</v>
       </c>
       <c r="I92" t="n">
-        <v>9.017807541409163e-06</v>
+        <v>9.017807541409165e-06</v>
       </c>
       <c r="J92" t="n">
         <v>2.151177459893121e-05</v>
@@ -5483,10 +5483,10 @@
         <v>0.001218113079817947</v>
       </c>
       <c r="C93" t="n">
-        <v>0.0009638096057019049</v>
+        <v>0.0009638096057019052</v>
       </c>
       <c r="D93" t="n">
-        <v>0.0005535583722732743</v>
+        <v>0.0005535583722732744</v>
       </c>
       <c r="E93" t="n">
         <v>0.0002633231258510241</v>
@@ -5495,13 +5495,13 @@
         <v>0.000182270130230995</v>
       </c>
       <c r="G93" t="n">
-        <v>2.845095863042478e-05</v>
+        <v>2.845095863042477e-05</v>
       </c>
       <c r="H93" t="n">
         <v>1.357270892638599e-05</v>
       </c>
       <c r="I93" t="n">
-        <v>9.778791192269459e-06</v>
+        <v>9.778791192269458e-06</v>
       </c>
       <c r="J93" t="n">
         <v>2.104201106769334e-05</v>
@@ -5516,7 +5516,7 @@
         <v>2.414525007204356e-06</v>
       </c>
       <c r="N93" t="n">
-        <v>7.122128570417619e-07</v>
+        <v>7.12212857041762e-07</v>
       </c>
       <c r="O93" t="n">
         <v>7.409878180333377e-08</v>
@@ -5538,16 +5538,16 @@
         <v>0.001223392443903345</v>
       </c>
       <c r="C94" t="n">
-        <v>0.0009687324723434824</v>
+        <v>0.0009687324723434821</v>
       </c>
       <c r="D94" t="n">
-        <v>0.0005700280482615842</v>
+        <v>0.0005700280482615841</v>
       </c>
       <c r="E94" t="n">
         <v>0.0002685477092112585</v>
       </c>
       <c r="F94" t="n">
-        <v>0.0001913875342668877</v>
+        <v>0.0001913875342668878</v>
       </c>
       <c r="G94" t="n">
         <v>3.172925592950623e-05</v>
@@ -5556,7 +5556,7 @@
         <v>1.374787868657315e-05</v>
       </c>
       <c r="I94" t="n">
-        <v>9.610345324850096e-06</v>
+        <v>9.610345324850095e-06</v>
       </c>
       <c r="J94" t="n">
         <v>2.122253110322755e-05</v>
@@ -5568,7 +5568,7 @@
         <v>1.367642082035777e-05</v>
       </c>
       <c r="M94" t="n">
-        <v>2.510443925889119e-06</v>
+        <v>2.51044392588912e-06</v>
       </c>
       <c r="N94" t="n">
         <v>4.540004440952185e-07</v>
@@ -5590,34 +5590,34 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.00123640377007429</v>
+        <v>0.001236403770074289</v>
       </c>
       <c r="C95" t="n">
-        <v>0.0009862553767234531</v>
+        <v>0.0009862553767234527</v>
       </c>
       <c r="D95" t="n">
-        <v>0.0005697893939936831</v>
+        <v>0.0005697893939936834</v>
       </c>
       <c r="E95" t="n">
         <v>0.0002753441091309228</v>
       </c>
       <c r="F95" t="n">
-        <v>0.0001899144670785241</v>
+        <v>0.000189914467078524</v>
       </c>
       <c r="G95" t="n">
-        <v>2.843204588492657e-05</v>
+        <v>2.843204588492658e-05</v>
       </c>
       <c r="H95" t="n">
         <v>1.242259441921298e-05</v>
       </c>
       <c r="I95" t="n">
-        <v>9.007860905876556e-06</v>
+        <v>9.007860905876553e-06</v>
       </c>
       <c r="J95" t="n">
         <v>2.146255353468278e-05</v>
       </c>
       <c r="K95" t="n">
-        <v>1.728403986352239e-05</v>
+        <v>1.728403986352238e-05</v>
       </c>
       <c r="L95" t="n">
         <v>1.277216607907631e-05</v>
@@ -5626,7 +5626,7 @@
         <v>2.330397383965461e-06</v>
       </c>
       <c r="N95" t="n">
-        <v>4.244758568207435e-07</v>
+        <v>4.244758568207434e-07</v>
       </c>
       <c r="O95" t="n">
         <v>6.521607801162105e-08</v>
@@ -5645,13 +5645,13 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.001214400374035062</v>
+        <v>0.001214400374035061</v>
       </c>
       <c r="C96" t="n">
-        <v>0.0009678571711242372</v>
+        <v>0.0009678571711242371</v>
       </c>
       <c r="D96" t="n">
-        <v>0.0005610520264992133</v>
+        <v>0.0005610520264992136</v>
       </c>
       <c r="E96" t="n">
         <v>0.0002639530509159248</v>
@@ -5660,13 +5660,13 @@
         <v>0.0001851638601521489</v>
       </c>
       <c r="G96" t="n">
-        <v>3.040189830147518e-05</v>
+        <v>3.040189830147517e-05</v>
       </c>
       <c r="H96" t="n">
         <v>1.386726217796386e-05</v>
       </c>
       <c r="I96" t="n">
-        <v>9.50962044520731e-06</v>
+        <v>9.509620445207311e-06</v>
       </c>
       <c r="J96" t="n">
         <v>2.125262829253618e-05</v>
@@ -5675,7 +5675,7 @@
         <v>1.675382623948599e-05</v>
       </c>
       <c r="L96" t="n">
-        <v>1.275004492952608e-05</v>
+        <v>1.275004492952609e-05</v>
       </c>
       <c r="M96" t="n">
         <v>2.372803471497839e-06</v>
@@ -5706,22 +5706,22 @@
         <v>0.001009478631473034</v>
       </c>
       <c r="D97" t="n">
-        <v>0.000591107729978316</v>
+        <v>0.0005911077299783158</v>
       </c>
       <c r="E97" t="n">
         <v>0.0002918553434705197</v>
       </c>
       <c r="F97" t="n">
-        <v>0.0001920917655108689</v>
+        <v>0.0001920917655108688</v>
       </c>
       <c r="G97" t="n">
-        <v>2.712484246808702e-05</v>
+        <v>2.712484246808701e-05</v>
       </c>
       <c r="H97" t="n">
         <v>8.305747670695093e-06</v>
       </c>
       <c r="I97" t="n">
-        <v>8.37360614221729e-06</v>
+        <v>8.373606142217288e-06</v>
       </c>
       <c r="J97" t="n">
         <v>2.045392357493081e-05</v>
@@ -5733,7 +5733,7 @@
         <v>1.623170400531149e-05</v>
       </c>
       <c r="M97" t="n">
-        <v>2.476061215805098e-06</v>
+        <v>2.476061215805099e-06</v>
       </c>
       <c r="N97" t="n">
         <v>4.625393635725288e-07</v>
@@ -5758,10 +5758,10 @@
         <v>0.001243428887111998</v>
       </c>
       <c r="C98" t="n">
-        <v>0.001010037278210594</v>
+        <v>0.001010037278210593</v>
       </c>
       <c r="D98" t="n">
-        <v>0.0005933955054579772</v>
+        <v>0.0005933955054579766</v>
       </c>
       <c r="E98" t="n">
         <v>0.0002908809616024845</v>
@@ -5813,10 +5813,10 @@
         <v>0.001243229375800049</v>
       </c>
       <c r="C99" t="n">
-        <v>0.001010547959439606</v>
+        <v>0.001010547959439607</v>
       </c>
       <c r="D99" t="n">
-        <v>0.0005942450297246014</v>
+        <v>0.0005942450297246009</v>
       </c>
       <c r="E99" t="n">
         <v>0.0002936187929806078</v>
@@ -5831,7 +5831,7 @@
         <v>8.78826092627567e-06</v>
       </c>
       <c r="I99" t="n">
-        <v>9.317692939486619e-06</v>
+        <v>9.317692939486621e-06</v>
       </c>
       <c r="J99" t="n">
         <v>2.075821882875601e-05</v>
@@ -5868,10 +5868,10 @@
         <v>0.001224424204078127</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0009894549864831791</v>
+        <v>0.0009894549864831795</v>
       </c>
       <c r="D100" t="n">
-        <v>0.0005843231764583777</v>
+        <v>0.0005843231764583776</v>
       </c>
       <c r="E100" t="n">
         <v>0.0002878872733129364</v>
@@ -5880,13 +5880,13 @@
         <v>0.0001854823475079824</v>
       </c>
       <c r="G100" t="n">
-        <v>3.000275248729798e-05</v>
+        <v>3.000275248729797e-05</v>
       </c>
       <c r="H100" t="n">
         <v>8.594224280439573e-06</v>
       </c>
       <c r="I100" t="n">
-        <v>8.477054514743167e-06</v>
+        <v>8.477054514743169e-06</v>
       </c>
       <c r="J100" t="n">
         <v>2.077384793215171e-05</v>
@@ -5898,7 +5898,7 @@
         <v>1.540114658333456e-05</v>
       </c>
       <c r="M100" t="n">
-        <v>2.276325901287971e-06</v>
+        <v>2.276325901287972e-06</v>
       </c>
       <c r="N100" t="n">
         <v>3.555902909210001e-07</v>
@@ -5926,10 +5926,10 @@
         <v>0.001010065872611721</v>
       </c>
       <c r="D101" t="n">
-        <v>0.000589782359613149</v>
+        <v>0.0005897823596131487</v>
       </c>
       <c r="E101" t="n">
-        <v>0.0002972577968400163</v>
+        <v>0.0002972577968400164</v>
       </c>
       <c r="F101" t="n">
         <v>0.0001918171481873006</v>
@@ -5941,7 +5941,7 @@
         <v>8.85217297124276e-06</v>
       </c>
       <c r="I101" t="n">
-        <v>9.233233334044428e-06</v>
+        <v>9.233233334044429e-06</v>
       </c>
       <c r="J101" t="n">
         <v>2.046962200470023e-05</v>
@@ -5953,7 +5953,7 @@
         <v>1.500532267342184e-05</v>
       </c>
       <c r="M101" t="n">
-        <v>2.297827499830417e-06</v>
+        <v>2.297827499830416e-06</v>
       </c>
       <c r="N101" t="n">
         <v>2.615051293349754e-07</v>
@@ -5981,7 +5981,7 @@
         <v>0.001006157247880849</v>
       </c>
       <c r="D102" t="n">
-        <v>0.0005902077487280802</v>
+        <v>0.00059020774872808</v>
       </c>
       <c r="E102" t="n">
         <v>0.0002880156805705588</v>
@@ -5996,13 +5996,13 @@
         <v>9.320007161648193e-06</v>
       </c>
       <c r="I102" t="n">
-        <v>8.645501837801665e-06</v>
+        <v>8.645501837801669e-06</v>
       </c>
       <c r="J102" t="n">
         <v>2.120000884445672e-05</v>
       </c>
       <c r="K102" t="n">
-        <v>1.647227631183039e-05</v>
+        <v>1.64722763118304e-05</v>
       </c>
       <c r="L102" t="n">
         <v>1.444664013947564e-05</v>
@@ -6030,13 +6030,13 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.001237697028597786</v>
+        <v>0.001237697028597788</v>
       </c>
       <c r="C103" t="n">
         <v>0.001007127296936323</v>
       </c>
       <c r="D103" t="n">
-        <v>0.0005821504702350958</v>
+        <v>0.0005821504702350962</v>
       </c>
       <c r="E103" t="n">
         <v>0.0002966482046324392</v>
@@ -6051,7 +6051,7 @@
         <v>1.041622653240662e-05</v>
       </c>
       <c r="I103" t="n">
-        <v>9.018401192032194e-06</v>
+        <v>9.018401192032192e-06</v>
       </c>
       <c r="J103" t="n">
         <v>2.0276591496805e-05</v>
@@ -6083,19 +6083,19 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.001239470718663824</v>
+        <v>0.001239470718663826</v>
       </c>
       <c r="C104" t="n">
         <v>0.001015108596401458</v>
       </c>
       <c r="D104" t="n">
-        <v>0.0005921505950543069</v>
+        <v>0.0005921505950543071</v>
       </c>
       <c r="E104" t="n">
-        <v>0.0002953083532076737</v>
+        <v>0.0002953083532076738</v>
       </c>
       <c r="F104" t="n">
-        <v>0.0001961717710081791</v>
+        <v>0.000196171771008179</v>
       </c>
       <c r="G104" t="n">
         <v>2.762556624852057e-05</v>
@@ -6110,7 +6110,7 @@
         <v>2.023890913079537e-05</v>
       </c>
       <c r="K104" t="n">
-        <v>1.681295740498247e-05</v>
+        <v>1.681295740498248e-05</v>
       </c>
       <c r="L104" t="n">
         <v>1.486930522804151e-05</v>
@@ -6138,13 +6138,13 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.001245094783342514</v>
+        <v>0.001245094783342515</v>
       </c>
       <c r="C105" t="n">
-        <v>0.001017168292726599</v>
+        <v>0.0010171682927266</v>
       </c>
       <c r="D105" t="n">
-        <v>0.0005858707263415544</v>
+        <v>0.000585870726341555</v>
       </c>
       <c r="E105" t="n">
         <v>0.0003013361102666489</v>
@@ -6159,7 +6159,7 @@
         <v>1.048960121910412e-05</v>
       </c>
       <c r="I105" t="n">
-        <v>8.877610244495405e-06</v>
+        <v>8.877610244495401e-06</v>
       </c>
       <c r="J105" t="n">
         <v>2.02846332070839e-05</v>
@@ -6202,7 +6202,7 @@
         <v>0.0005907738276034113</v>
       </c>
       <c r="E106" t="n">
-        <v>0.0002899311207595873</v>
+        <v>0.0002899311207595874</v>
       </c>
       <c r="F106" t="n">
         <v>0.0001947632745084014</v>
@@ -6254,10 +6254,10 @@
         <v>0.001025056537481052</v>
       </c>
       <c r="D107" t="n">
-        <v>0.0005933652801908319</v>
+        <v>0.0005933652801908316</v>
       </c>
       <c r="E107" t="n">
-        <v>0.0002935139055580396</v>
+        <v>0.0002935139055580397</v>
       </c>
       <c r="F107" t="n">
         <v>0.0001948572141722064</v>
@@ -6281,10 +6281,10 @@
         <v>1.540442562506303e-05</v>
       </c>
       <c r="M107" t="n">
-        <v>2.464641608923581e-06</v>
+        <v>2.464641608923582e-06</v>
       </c>
       <c r="N107" t="n">
-        <v>5.308095272734793e-07</v>
+        <v>5.308095272734792e-07</v>
       </c>
       <c r="O107" t="n">
         <v>6.503592848833394e-08</v>
@@ -6303,13 +6303,13 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.001237503542587311</v>
+        <v>0.001237503542587313</v>
       </c>
       <c r="C108" t="n">
         <v>0.001009477342821114</v>
       </c>
       <c r="D108" t="n">
-        <v>0.0005900100415158605</v>
+        <v>0.0005900100415158604</v>
       </c>
       <c r="E108" t="n">
         <v>0.0002931775715733849</v>
@@ -6318,7 +6318,7 @@
         <v>0.0001958900949752632</v>
       </c>
       <c r="G108" t="n">
-        <v>2.840264586824747e-05</v>
+        <v>2.840264586824746e-05</v>
       </c>
       <c r="H108" t="n">
         <v>1.248740658033015e-05</v>
@@ -6339,7 +6339,7 @@
         <v>2.597741717479367e-06</v>
       </c>
       <c r="N108" t="n">
-        <v>4.284279235722335e-07</v>
+        <v>4.284279235722336e-07</v>
       </c>
       <c r="O108" t="n">
         <v>6.310743329113018e-08</v>
@@ -6358,13 +6358,13 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.001288988403303318</v>
+        <v>0.001288988403303319</v>
       </c>
       <c r="C109" t="n">
-        <v>0.001044088546000763</v>
+        <v>0.001044088546000762</v>
       </c>
       <c r="D109" t="n">
-        <v>0.000590140449504905</v>
+        <v>0.0005901404495049052</v>
       </c>
       <c r="E109" t="n">
         <v>0.0003022097438247084</v>
@@ -6391,7 +6391,7 @@
         <v>1.425032461675525e-05</v>
       </c>
       <c r="M109" t="n">
-        <v>2.455266196565921e-06</v>
+        <v>2.45526619656592e-06</v>
       </c>
       <c r="N109" t="n">
         <v>3.560971539608313e-07</v>
@@ -6413,13 +6413,13 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.001279679014722205</v>
+        <v>0.001279679014722206</v>
       </c>
       <c r="C110" t="n">
         <v>0.001038453548806432</v>
       </c>
       <c r="D110" t="n">
-        <v>0.0005929363630136867</v>
+        <v>0.0005929363630136863</v>
       </c>
       <c r="E110" t="n">
         <v>0.0003008691239100288</v>
@@ -6428,13 +6428,13 @@
         <v>0.0002000415619633553</v>
       </c>
       <c r="G110" t="n">
-        <v>2.735886841104184e-05</v>
+        <v>2.735886841104183e-05</v>
       </c>
       <c r="H110" t="n">
         <v>1.129957443337404e-05</v>
       </c>
       <c r="I110" t="n">
-        <v>8.737482239465382e-06</v>
+        <v>8.73748223946538e-06</v>
       </c>
       <c r="J110" t="n">
         <v>2.018739327280161e-05</v>
@@ -6474,7 +6474,7 @@
         <v>0.00103078447000247</v>
       </c>
       <c r="D111" t="n">
-        <v>0.0005868962083948631</v>
+        <v>0.0005868962083948626</v>
       </c>
       <c r="E111" t="n">
         <v>0.0002971122246850985</v>
@@ -6544,7 +6544,7 @@
         <v>9.286100760984489e-06</v>
       </c>
       <c r="I112" t="n">
-        <v>8.758141591019113e-06</v>
+        <v>8.75814159101911e-06</v>
       </c>
       <c r="J112" t="n">
         <v>2.014537923670973e-05</v>
@@ -6578,7 +6578,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.001307240600822645</v>
+        <v>0.001307240600822644</v>
       </c>
       <c r="C113" t="n">
         <v>0.001067951613502765</v>
@@ -6587,19 +6587,19 @@
         <v>0.000606707359252503</v>
       </c>
       <c r="E113" t="n">
-        <v>0.0003139541131491072</v>
+        <v>0.0003139541131491073</v>
       </c>
       <c r="F113" t="n">
         <v>0.0002067862033186216</v>
       </c>
       <c r="G113" t="n">
-        <v>2.525939137873163e-05</v>
+        <v>2.525939137873165e-05</v>
       </c>
       <c r="H113" t="n">
         <v>9.126292610060131e-06</v>
       </c>
       <c r="I113" t="n">
-        <v>8.581070237578802e-06</v>
+        <v>8.581070237578804e-06</v>
       </c>
       <c r="J113" t="n">
         <v>2.035577584582205e-05</v>
@@ -6639,16 +6639,16 @@
         <v>0.001068043301399413</v>
       </c>
       <c r="D114" t="n">
-        <v>0.0005980268106675347</v>
+        <v>0.0005980268106675349</v>
       </c>
       <c r="E114" t="n">
-        <v>0.0003242014808437753</v>
+        <v>0.0003242014808437754</v>
       </c>
       <c r="F114" t="n">
         <v>0.0002009907694992277</v>
       </c>
       <c r="G114" t="n">
-        <v>2.535797146999705e-05</v>
+        <v>2.535797146999704e-05</v>
       </c>
       <c r="H114" t="n">
         <v>9.494015627487198e-06</v>
@@ -6669,7 +6669,7 @@
         <v>2.371016050783024e-06</v>
       </c>
       <c r="N114" t="n">
-        <v>3.168016409551447e-07</v>
+        <v>3.168016409551448e-07</v>
       </c>
       <c r="O114" t="n">
         <v>5.515893750302788e-08</v>
@@ -6688,19 +6688,19 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.001261950283330128</v>
+        <v>0.001261950283330127</v>
       </c>
       <c r="C115" t="n">
         <v>0.001035321968832714</v>
       </c>
       <c r="D115" t="n">
-        <v>0.0005926686391573927</v>
+        <v>0.0005926686391573929</v>
       </c>
       <c r="E115" t="n">
         <v>0.0003034643863215369</v>
       </c>
       <c r="F115" t="n">
-        <v>0.0001943060470249355</v>
+        <v>0.0001943060470249356</v>
       </c>
       <c r="G115" t="n">
         <v>2.765254640766942e-05</v>
@@ -6709,7 +6709,7 @@
         <v>1.029767006604482e-05</v>
       </c>
       <c r="I115" t="n">
-        <v>9.335515246927961e-06</v>
+        <v>9.33551524692796e-06</v>
       </c>
       <c r="J115" t="n">
         <v>1.923630689016146e-05</v>
@@ -6718,7 +6718,7 @@
         <v>1.668502065240609e-05</v>
       </c>
       <c r="L115" t="n">
-        <v>1.427023761416494e-05</v>
+        <v>1.427023761416495e-05</v>
       </c>
       <c r="M115" t="n">
         <v>2.262934236006005e-06</v>
@@ -6743,16 +6743,16 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.001274852726501692</v>
+        <v>0.001274852726501693</v>
       </c>
       <c r="C116" t="n">
         <v>0.001045824824155983</v>
       </c>
       <c r="D116" t="n">
-        <v>0.0006050491151323017</v>
+        <v>0.0006050491151323015</v>
       </c>
       <c r="E116" t="n">
-        <v>0.000301247821719607</v>
+        <v>0.0003012478217196069</v>
       </c>
       <c r="F116" t="n">
         <v>0.0002002114892733328</v>
@@ -6764,7 +6764,7 @@
         <v>1.047850413573022e-05</v>
       </c>
       <c r="I116" t="n">
-        <v>9.164085460532355e-06</v>
+        <v>9.164085460532359e-06</v>
       </c>
       <c r="J116" t="n">
         <v>1.968306510602948e-05</v>
@@ -6798,7 +6798,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.001343127625318067</v>
+        <v>0.001343127625318068</v>
       </c>
       <c r="C117" t="n">
         <v>0.001049228527925733</v>
@@ -6807,13 +6807,13 @@
         <v>0.0006111597539049073</v>
       </c>
       <c r="E117" t="n">
-        <v>0.0003005509783103488</v>
+        <v>0.0003005509783103489</v>
       </c>
       <c r="F117" t="n">
-        <v>0.0001951968494241513</v>
+        <v>0.0001951968494241512</v>
       </c>
       <c r="G117" t="n">
-        <v>2.791500541266006e-05</v>
+        <v>2.791500541266007e-05</v>
       </c>
       <c r="H117" t="n">
         <v>1.166136709189628e-05</v>
@@ -6857,7 +6857,7 @@
         <v>0.001029422743105408</v>
       </c>
       <c r="D118" t="n">
-        <v>0.0005961861132289826</v>
+        <v>0.0005961861132289827</v>
       </c>
       <c r="E118" t="n">
         <v>0.0002883706791967664</v>
@@ -6872,7 +6872,7 @@
         <v>1.105060925044967e-05</v>
       </c>
       <c r="I118" t="n">
-        <v>8.69578167318435e-06</v>
+        <v>8.695781673184348e-06</v>
       </c>
       <c r="J118" t="n">
         <v>1.978581728393647e-05</v>
@@ -6881,13 +6881,13 @@
         <v>1.690790218751646e-05</v>
       </c>
       <c r="L118" t="n">
-        <v>1.437542311413969e-05</v>
+        <v>1.43754231141397e-05</v>
       </c>
       <c r="M118" t="n">
         <v>2.257649001698841e-06</v>
       </c>
       <c r="N118" t="n">
-        <v>3.659316311770611e-07</v>
+        <v>3.659316311770612e-07</v>
       </c>
       <c r="O118" t="n">
         <v>6.818183265222701e-08</v>
@@ -6909,16 +6909,16 @@
         <v>0.001257302077167623</v>
       </c>
       <c r="C119" t="n">
-        <v>0.00102804288837091</v>
+        <v>0.001028042888370911</v>
       </c>
       <c r="D119" t="n">
-        <v>0.0005955559121688798</v>
+        <v>0.0005955559121688797</v>
       </c>
       <c r="E119" t="n">
         <v>0.0002934493354598253</v>
       </c>
       <c r="F119" t="n">
-        <v>0.0001967459237552531</v>
+        <v>0.000196745923755253</v>
       </c>
       <c r="G119" t="n">
         <v>2.711934681645401e-05</v>
@@ -6927,7 +6927,7 @@
         <v>1.041752623339936e-05</v>
       </c>
       <c r="I119" t="n">
-        <v>9.492231304769744e-06</v>
+        <v>9.492231304769741e-06</v>
       </c>
       <c r="J119" t="n">
         <v>1.992937771689059e-05</v>
@@ -6939,7 +6939,7 @@
         <v>1.4507793067719e-05</v>
       </c>
       <c r="M119" t="n">
-        <v>2.2561630182314e-06</v>
+        <v>2.256163018231401e-06</v>
       </c>
       <c r="N119" t="n">
         <v>9.253761387004203e-07</v>
@@ -6961,16 +6961,16 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.001266997785620201</v>
+        <v>0.001266997785620202</v>
       </c>
       <c r="C120" t="n">
         <v>0.001035915855783454</v>
       </c>
       <c r="D120" t="n">
-        <v>0.0005979156105338961</v>
+        <v>0.0005979156105338963</v>
       </c>
       <c r="E120" t="n">
-        <v>0.0002964088463657096</v>
+        <v>0.0002964088463657097</v>
       </c>
       <c r="F120" t="n">
         <v>0.000198566327204517</v>
@@ -6982,7 +6982,7 @@
         <v>1.096010032960748e-05</v>
       </c>
       <c r="I120" t="n">
-        <v>8.834219036474206e-06</v>
+        <v>8.834219036474204e-06</v>
       </c>
       <c r="J120" t="n">
         <v>2.008260341166297e-05</v>

</xml_diff>